<commit_message>
Feature/new summary reports types
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/summaryReportForm1.xlsx
+++ b/src/main/resources/templates/summaryReportForm1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F78BF3A-336A-429E-A23A-4C969CE9241F}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1AE005B-2035-4100-BBF6-1787ED9117FD}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,9 +49,6 @@
     <t>из них по культурам</t>
   </si>
   <si>
-    <t>Кр.т.гибель озимых, га</t>
-  </si>
-  <si>
     <t>СЕВ всего, га</t>
   </si>
   <si>
@@ -572,6 +569,9 @@
   </si>
   <si>
     <t>$header_reportDate</t>
+  </si>
+  <si>
+    <t>Кр.т. гибель озимых, га</t>
   </si>
 </sst>
 </file>
@@ -605,11 +605,6 @@
       <charset val="204"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Arial Cyr"/>
-      <charset val="204"/>
-    </font>
-    <font>
       <sz val="10"/>
       <name val="Arial Cyr"/>
       <charset val="204"/>
@@ -631,9 +626,18 @@
     </font>
     <font>
       <b/>
-      <sz val="9"/>
-      <name val="Arial Cyr"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1001,13 +1005,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1016,10 +1017,10 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1028,78 +1029,48 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1115,14 +1086,47 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1414,22 +1418,22 @@
   <sheetData>
     <row r="1" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
       <c r="P1" s="3"/>
       <c r="Q1" s="3"/>
       <c r="R1" s="3"/>
@@ -1483,22 +1487,22 @@
     </row>
     <row r="2" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
@@ -1563,7 +1567,7 @@
         <v>2</v>
       </c>
       <c r="J3" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -1755,924 +1759,961 @@
       <c r="BL5" s="2"/>
       <c r="BM5" s="2"/>
     </row>
-    <row r="6" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="31" t="s">
+    <row r="6" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="49" t="s">
+      <c r="C6" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="51" t="s">
+      <c r="D6" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="32" t="s">
+      <c r="E6" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="32" t="s">
+      <c r="F6" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
-      <c r="J6" s="32"/>
-      <c r="K6" s="33" t="s">
+      <c r="G6" s="42"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
+      <c r="K6" s="35" t="s">
+        <v>183</v>
+      </c>
+      <c r="L6" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="L6" s="31" t="s">
+      <c r="M6" s="42"/>
+      <c r="N6" s="42"/>
+      <c r="O6" s="42"/>
+      <c r="P6" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="M6" s="32"/>
-      <c r="N6" s="32"/>
-      <c r="O6" s="32"/>
-      <c r="P6" s="41" t="s">
+      <c r="Q6" s="49"/>
+      <c r="R6" s="49"/>
+      <c r="S6" s="49"/>
+      <c r="T6" s="49"/>
+      <c r="U6" s="49"/>
+      <c r="V6" s="49"/>
+      <c r="W6" s="49"/>
+      <c r="X6" s="49"/>
+      <c r="Y6" s="49"/>
+      <c r="Z6" s="49"/>
+      <c r="AA6" s="49"/>
+      <c r="AB6" s="49"/>
+      <c r="AC6" s="49"/>
+      <c r="AD6" s="49"/>
+      <c r="AE6" s="49"/>
+      <c r="AF6" s="49"/>
+      <c r="AG6" s="49"/>
+      <c r="AH6" s="49"/>
+      <c r="AI6" s="49"/>
+      <c r="AJ6" s="49"/>
+      <c r="AK6" s="49"/>
+      <c r="AL6" s="49"/>
+      <c r="AM6" s="49"/>
+      <c r="AN6" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="Q6" s="42"/>
-      <c r="R6" s="42"/>
-      <c r="S6" s="42"/>
-      <c r="T6" s="42"/>
-      <c r="U6" s="42"/>
-      <c r="V6" s="42"/>
-      <c r="W6" s="42"/>
-      <c r="X6" s="42"/>
-      <c r="Y6" s="42"/>
-      <c r="Z6" s="42"/>
-      <c r="AA6" s="42"/>
-      <c r="AB6" s="42"/>
-      <c r="AC6" s="42"/>
-      <c r="AD6" s="42"/>
-      <c r="AE6" s="42"/>
-      <c r="AF6" s="42"/>
-      <c r="AG6" s="42"/>
-      <c r="AH6" s="42"/>
-      <c r="AI6" s="42"/>
-      <c r="AJ6" s="42"/>
-      <c r="AK6" s="42"/>
-      <c r="AL6" s="42"/>
-      <c r="AM6" s="42"/>
-      <c r="AN6" s="31" t="s">
+      <c r="AO6" s="42"/>
+      <c r="AP6" s="42"/>
+      <c r="AQ6" s="42"/>
+      <c r="AR6" s="35"/>
+      <c r="AS6" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="AO6" s="32"/>
-      <c r="AP6" s="32"/>
-      <c r="AQ6" s="32"/>
-      <c r="AR6" s="33"/>
-      <c r="AS6" s="43" t="s">
+      <c r="AT6" s="42"/>
+      <c r="AU6" s="42"/>
+      <c r="AV6" s="42"/>
+      <c r="AW6" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="AT6" s="32"/>
-      <c r="AU6" s="32"/>
-      <c r="AV6" s="32"/>
-      <c r="AW6" s="31" t="s">
+      <c r="AX6" s="42"/>
+      <c r="AY6" s="42"/>
+      <c r="AZ6" s="35"/>
+      <c r="BA6" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="AX6" s="32"/>
-      <c r="AY6" s="32"/>
-      <c r="AZ6" s="33"/>
-      <c r="BA6" s="44" t="s">
+      <c r="BB6" s="51"/>
+      <c r="BC6" s="51"/>
+      <c r="BD6" s="52"/>
+      <c r="BE6" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="BB6" s="44"/>
-      <c r="BC6" s="44"/>
-      <c r="BD6" s="45"/>
-      <c r="BE6" s="42" t="s">
+      <c r="BF6" s="49"/>
+      <c r="BG6" s="49"/>
+      <c r="BH6" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="BF6" s="42"/>
-      <c r="BG6" s="42"/>
-      <c r="BH6" s="31" t="s">
+      <c r="BI6" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="BI6" s="31" t="s">
+      <c r="BJ6" s="42"/>
+      <c r="BK6" s="35"/>
+      <c r="BL6" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="BJ6" s="32"/>
-      <c r="BK6" s="33"/>
-      <c r="BL6" s="32" t="s">
+      <c r="BM6" s="42"/>
+    </row>
+    <row r="7" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="33"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="BM6" s="32"/>
+      <c r="G7" s="43" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="K7" s="36"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="30"/>
+      <c r="N7" s="30"/>
+      <c r="O7" s="30"/>
+      <c r="P7" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q7" s="30"/>
+      <c r="R7" s="30"/>
+      <c r="S7" s="30"/>
+      <c r="T7" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="U7" s="30"/>
+      <c r="V7" s="30"/>
+      <c r="W7" s="30"/>
+      <c r="X7" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y7" s="47"/>
+      <c r="Z7" s="47"/>
+      <c r="AA7" s="46"/>
+      <c r="AB7" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC7" s="30"/>
+      <c r="AD7" s="30"/>
+      <c r="AE7" s="30"/>
+      <c r="AF7" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="AG7" s="30"/>
+      <c r="AH7" s="30"/>
+      <c r="AI7" s="30"/>
+      <c r="AJ7" s="47" t="s">
+        <v>29</v>
+      </c>
+      <c r="AK7" s="47"/>
+      <c r="AL7" s="47"/>
+      <c r="AM7" s="47"/>
+      <c r="AN7" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="AO7" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="AP7" s="30"/>
+      <c r="AQ7" s="30"/>
+      <c r="AR7" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="AS7" s="46" t="s">
+        <v>30</v>
+      </c>
+      <c r="AT7" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="AU7" s="30"/>
+      <c r="AV7" s="30"/>
+      <c r="AW7" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="AX7" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="AY7" s="30"/>
+      <c r="AZ7" s="36"/>
+      <c r="BA7" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="BB7" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="BC7" s="54" t="s">
+        <v>35</v>
+      </c>
+      <c r="BD7" s="55" t="s">
+        <v>36</v>
+      </c>
+      <c r="BE7" s="53" t="s">
+        <v>37</v>
+      </c>
+      <c r="BF7" s="53"/>
+      <c r="BG7" s="53"/>
+      <c r="BH7" s="33"/>
+      <c r="BI7" s="33" t="s">
+        <v>38</v>
+      </c>
+      <c r="BJ7" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="BK7" s="36"/>
+      <c r="BL7" s="30"/>
+      <c r="BM7" s="30"/>
     </row>
-    <row r="7" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="28"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="50"/>
-      <c r="D7" s="52"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" s="39" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="J7" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="K7" s="36"/>
-      <c r="L7" s="28"/>
-      <c r="M7" s="29"/>
-      <c r="N7" s="29"/>
-      <c r="O7" s="29"/>
-      <c r="P7" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q7" s="29"/>
-      <c r="R7" s="29"/>
-      <c r="S7" s="29"/>
-      <c r="T7" s="29" t="s">
-        <v>26</v>
-      </c>
-      <c r="U7" s="29"/>
-      <c r="V7" s="29"/>
-      <c r="W7" s="29"/>
-      <c r="X7" s="38" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y7" s="30"/>
-      <c r="Z7" s="30"/>
-      <c r="AA7" s="37"/>
-      <c r="AB7" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="AC7" s="29"/>
-      <c r="AD7" s="29"/>
-      <c r="AE7" s="29"/>
-      <c r="AF7" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="AG7" s="29"/>
-      <c r="AH7" s="29"/>
-      <c r="AI7" s="29"/>
-      <c r="AJ7" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="AK7" s="30"/>
-      <c r="AL7" s="30"/>
-      <c r="AM7" s="30"/>
-      <c r="AN7" s="28" t="s">
+    <row r="8" spans="1:65" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="33"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="AO7" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="AP7" s="29"/>
-      <c r="AQ7" s="29"/>
-      <c r="AR7" s="36" t="s">
-        <v>33</v>
-      </c>
-      <c r="AS7" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="AT7" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="AU7" s="29"/>
-      <c r="AV7" s="29"/>
-      <c r="AW7" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="AX7" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="AY7" s="29"/>
-      <c r="AZ7" s="36"/>
-      <c r="BA7" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="BB7" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="BC7" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="BD7" s="35" t="s">
-        <v>37</v>
-      </c>
-      <c r="BE7" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="BF7" s="27"/>
-      <c r="BG7" s="27"/>
-      <c r="BH7" s="28"/>
-      <c r="BI7" s="28" t="s">
-        <v>39</v>
-      </c>
-      <c r="BJ7" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="BK7" s="36"/>
-      <c r="BL7" s="29"/>
-      <c r="BM7" s="29"/>
-    </row>
-    <row r="8" spans="1:65" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="28"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="50"/>
-      <c r="D8" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
       <c r="K8" s="36"/>
       <c r="L8" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M8" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="M8" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="N8" s="29"/>
+      <c r="N8" s="30"/>
       <c r="O8" s="8"/>
       <c r="P8" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q8" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="Q8" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="R8" s="29"/>
+      <c r="R8" s="30"/>
       <c r="S8" s="8"/>
       <c r="T8" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="U8" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="V8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="W8" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="V8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="W8" s="8" t="s">
-        <v>42</v>
-      </c>
       <c r="X8" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y8" s="45" t="s">
         <v>31</v>
       </c>
-      <c r="Y8" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="Z8" s="37"/>
+      <c r="Z8" s="46"/>
       <c r="AA8" s="8"/>
       <c r="AB8" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC8" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="AC8" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="AD8" s="29"/>
+      <c r="AD8" s="30"/>
       <c r="AE8" s="8"/>
       <c r="AF8" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG8" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="AG8" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="AH8" s="29"/>
+      <c r="AH8" s="30"/>
       <c r="AI8" s="8"/>
       <c r="AJ8" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="AK8" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="AK8" s="8" t="s">
+      <c r="AL8" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="AL8" s="8" t="s">
+      <c r="AM8" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="AM8" s="9" t="s">
+      <c r="AN8" s="33"/>
+      <c r="AO8" s="30"/>
+      <c r="AP8" s="30"/>
+      <c r="AQ8" s="30"/>
+      <c r="AR8" s="36"/>
+      <c r="AS8" s="46"/>
+      <c r="AT8" s="30"/>
+      <c r="AU8" s="30"/>
+      <c r="AV8" s="30"/>
+      <c r="AW8" s="33"/>
+      <c r="AX8" s="30"/>
+      <c r="AY8" s="30"/>
+      <c r="AZ8" s="36"/>
+      <c r="BA8" s="30"/>
+      <c r="BB8" s="30"/>
+      <c r="BC8" s="54"/>
+      <c r="BD8" s="55"/>
+      <c r="BE8" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="AN8" s="28"/>
-      <c r="AO8" s="29"/>
-      <c r="AP8" s="29"/>
-      <c r="AQ8" s="29"/>
-      <c r="AR8" s="36"/>
-      <c r="AS8" s="37"/>
-      <c r="AT8" s="29"/>
-      <c r="AU8" s="29"/>
-      <c r="AV8" s="29"/>
-      <c r="AW8" s="28"/>
-      <c r="AX8" s="29"/>
-      <c r="AY8" s="29"/>
-      <c r="AZ8" s="36"/>
-      <c r="BA8" s="29"/>
-      <c r="BB8" s="29"/>
-      <c r="BC8" s="34"/>
-      <c r="BD8" s="35"/>
-      <c r="BE8" s="8" t="s">
+      <c r="BF8" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="BF8" s="8" t="s">
+      <c r="BG8" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="BG8" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="BH8" s="28"/>
-      <c r="BI8" s="28"/>
-      <c r="BJ8" s="29"/>
+      <c r="BH8" s="33"/>
+      <c r="BI8" s="33"/>
+      <c r="BJ8" s="30"/>
       <c r="BK8" s="36"/>
       <c r="BL8" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="BM8" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:65" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="47"/>
-      <c r="B9" s="48"/>
-      <c r="C9" s="50"/>
+      <c r="A9" s="34"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="39"/>
       <c r="D9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="L9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="M9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="N9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="O9" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="P9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="R9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="S9" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="T9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="U9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="V9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="W9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="X9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA9" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AC9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="AD9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AE9" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="AF9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AG9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="AH9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AI9" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="AJ9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AL9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AM9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AN9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AO9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="AP9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AQ9" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR9" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="AS9" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="AT9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="AU9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AV9" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="AW9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="AX9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="AY9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AZ9" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="BA9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BB9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BC9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BD9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BE9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BF9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BG9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BH9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BI9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BJ9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BK9" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="BL9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BM9" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:65" s="20" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="J9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="L9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="M9" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="O9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="P9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q9" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="R9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="S9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="T9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="U9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="V9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="W9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="X9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y9" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="Z9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AA9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="AB9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC9" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="AF9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AG9" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="AH9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="AJ9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AK9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AL9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AM9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AN9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO9" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="AP9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="AR9" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="AS9" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="AT9" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="AU9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AV9" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="AW9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="AX9" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="AY9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="AZ9" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="BA9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="BB9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="BC9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="BD9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="BE9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="BF9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="BG9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="BH9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="BI9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="BJ9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="BK9" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="BL9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="BM9" s="10" t="s">
-        <v>53</v>
+      <c r="B10" s="26"/>
+      <c r="C10" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="I10" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="J10" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="K10" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="L10" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="M10" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="N10" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="O10" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="P10" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q10" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="R10" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="S10" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="T10" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="U10" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="V10" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="W10" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="X10" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="Y10" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="Z10" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="AA10" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="AB10" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="AC10" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="AD10" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="AE10" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="AF10" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="AG10" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="AH10" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="AI10" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="AJ10" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="AK10" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="AL10" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AM10" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="AN10" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="AO10" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="AP10" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="AQ10" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="AR10" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="AS10" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="AT10" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="AU10" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="AV10" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="AW10" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="AX10" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="AY10" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="AZ10" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="BA10" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="BB10" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="BC10" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="BD10" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="BE10" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="BF10" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="BG10" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="BH10" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="BI10" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="BJ10" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="BK10" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="BL10" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="BM10" s="19" t="s">
+        <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:65" s="21" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="54"/>
-      <c r="C10" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="F10" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="G10" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="I10" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="J10" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="K10" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="L10" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="M10" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="N10" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="O10" s="17" t="s">
-        <v>109</v>
-      </c>
-      <c r="P10" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q10" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="R10" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="S10" s="18" t="s">
-        <v>110</v>
-      </c>
-      <c r="T10" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="U10" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="V10" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="W10" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="X10" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="Y10" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="Z10" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="AA10" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="AB10" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="AC10" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="AD10" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="AE10" s="18" t="s">
-        <v>182</v>
-      </c>
-      <c r="AF10" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="AG10" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="AH10" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="AI10" s="18" t="s">
-        <v>112</v>
-      </c>
-      <c r="AJ10" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="AK10" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="AL10" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="AM10" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="AN10" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="AO10" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP10" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="AQ10" s="17" t="s">
-        <v>113</v>
-      </c>
-      <c r="AR10" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="AS10" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="AT10" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="AU10" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="AV10" s="17" t="s">
-        <v>114</v>
-      </c>
-      <c r="AW10" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AX10" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="AY10" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="AZ10" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="BA10" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="BB10" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="BC10" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="BD10" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="BE10" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="BF10" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="BG10" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="BH10" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="BI10" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="BJ10" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="BK10" s="18" t="s">
+    <row r="11" spans="1:65" s="25" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="BL10" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="BM10" s="20" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="11" spans="1:65" s="26" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="53" t="s">
+      <c r="B11" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="55" t="s">
+      <c r="C11" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="D11" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="E11" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="E11" s="22" t="s">
+      <c r="F11" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="F11" s="22" t="s">
+      <c r="G11" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="G11" s="22" t="s">
+      <c r="H11" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="H11" s="22" t="s">
+      <c r="I11" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="I11" s="22" t="s">
+      <c r="J11" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="J11" s="22" t="s">
+      <c r="K11" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="K11" s="22" t="s">
+      <c r="L11" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="L11" s="22" t="s">
+      <c r="M11" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="M11" s="22" t="s">
+      <c r="N11" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="N11" s="22" t="s">
+      <c r="O11" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="O11" s="23" t="s">
+      <c r="P11" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="P11" s="22" t="s">
+      <c r="Q11" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="Q11" s="22" t="s">
+      <c r="R11" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="R11" s="22" t="s">
+      <c r="S11" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="S11" s="24" t="s">
+      <c r="T11" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="T11" s="22" t="s">
+      <c r="U11" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="U11" s="22" t="s">
+      <c r="V11" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="V11" s="22" t="s">
+      <c r="W11" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="W11" s="22" t="s">
+      <c r="X11" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="X11" s="22" t="s">
+      <c r="Y11" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="Y11" s="22" t="s">
+      <c r="Z11" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="Z11" s="22" t="s">
+      <c r="AA11" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="AA11" s="24" t="s">
+      <c r="AB11" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="AC11" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="AB11" s="22" t="s">
+      <c r="AD11" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="AC11" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="AD11" s="22" t="s">
+      <c r="AE11" s="23" t="s">
         <v>146</v>
       </c>
-      <c r="AE11" s="24" t="s">
+      <c r="AF11" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="AF11" s="22" t="s">
+      <c r="AG11" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="AG11" s="22" t="s">
+      <c r="AH11" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="AH11" s="22" t="s">
+      <c r="AI11" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="AI11" s="24" t="s">
+      <c r="AJ11" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="AJ11" s="22" t="s">
+      <c r="AK11" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="AK11" s="22" t="s">
+      <c r="AL11" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="AL11" s="22" t="s">
+      <c r="AM11" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="AM11" s="22" t="s">
+      <c r="AN11" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="AN11" s="22" t="s">
+      <c r="AO11" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="AO11" s="22" t="s">
+      <c r="AP11" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="AP11" s="22" t="s">
+      <c r="AQ11" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="AQ11" s="23" t="s">
+      <c r="AR11" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="AR11" s="22" t="s">
+      <c r="AS11" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="AS11" s="22" t="s">
+      <c r="AT11" s="21" t="s">
         <v>161</v>
       </c>
-      <c r="AT11" s="22" t="s">
+      <c r="AU11" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="AU11" s="22" t="s">
+      <c r="AV11" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="AV11" s="23" t="s">
+      <c r="AW11" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="AW11" s="22" t="s">
+      <c r="AX11" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="AX11" s="22" t="s">
+      <c r="AY11" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="AY11" s="22" t="s">
+      <c r="AZ11" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="AZ11" s="24" t="s">
+      <c r="BA11" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="BA11" s="22" t="s">
+      <c r="BB11" s="21" t="s">
         <v>169</v>
       </c>
-      <c r="BB11" s="22" t="s">
+      <c r="BC11" s="21" t="s">
         <v>170</v>
       </c>
-      <c r="BC11" s="22" t="s">
+      <c r="BD11" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="BD11" s="22" t="s">
+      <c r="BE11" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="BE11" s="22" t="s">
+      <c r="BF11" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="BF11" s="22" t="s">
+      <c r="BG11" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="BG11" s="22" t="s">
+      <c r="BH11" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="BH11" s="22" t="s">
+      <c r="BI11" s="21" t="s">
         <v>176</v>
       </c>
-      <c r="BI11" s="22" t="s">
+      <c r="BJ11" s="21" t="s">
         <v>177</v>
       </c>
-      <c r="BJ11" s="22" t="s">
+      <c r="BK11" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="BK11" s="24" t="s">
+      <c r="BL11" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="BL11" s="22" t="s">
+      <c r="BM11" s="21" t="s">
         <v>180</v>
-      </c>
-      <c r="BM11" s="22" t="s">
-        <v>181</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="53">
+    <mergeCell ref="BE7:BG7"/>
+    <mergeCell ref="BI7:BI8"/>
+    <mergeCell ref="BJ7:BJ8"/>
+    <mergeCell ref="AW7:AW8"/>
+    <mergeCell ref="AB7:AE7"/>
+    <mergeCell ref="AF7:AI7"/>
+    <mergeCell ref="AJ7:AM7"/>
+    <mergeCell ref="AN7:AN8"/>
+    <mergeCell ref="AO7:AP8"/>
+    <mergeCell ref="BH6:BH8"/>
+    <mergeCell ref="BI6:BK6"/>
+    <mergeCell ref="BA7:BA8"/>
+    <mergeCell ref="BB7:BB8"/>
+    <mergeCell ref="BC7:BC8"/>
+    <mergeCell ref="BD7:BD8"/>
+    <mergeCell ref="AQ7:AQ8"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="AC8:AD8"/>
+    <mergeCell ref="AG8:AH8"/>
+    <mergeCell ref="P7:S7"/>
+    <mergeCell ref="T7:W7"/>
+    <mergeCell ref="AX7:AY8"/>
+    <mergeCell ref="AZ7:AZ8"/>
+    <mergeCell ref="Y8:Z8"/>
+    <mergeCell ref="X7:AA7"/>
+    <mergeCell ref="BL6:BM7"/>
+    <mergeCell ref="P6:AM6"/>
+    <mergeCell ref="AN6:AR6"/>
+    <mergeCell ref="AS6:AV6"/>
+    <mergeCell ref="AW6:AZ6"/>
+    <mergeCell ref="BA6:BD6"/>
+    <mergeCell ref="BE6:BG6"/>
+    <mergeCell ref="BK7:BK8"/>
+    <mergeCell ref="AR7:AR8"/>
+    <mergeCell ref="AS7:AS8"/>
+    <mergeCell ref="AT7:AU8"/>
+    <mergeCell ref="AV7:AV8"/>
     <mergeCell ref="M8:N8"/>
     <mergeCell ref="B1:O1"/>
     <mergeCell ref="B2:O2"/>
@@ -2689,45 +2730,8 @@
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="J7:J8"/>
-    <mergeCell ref="AX7:AY8"/>
-    <mergeCell ref="AZ7:AZ8"/>
-    <mergeCell ref="Y8:Z8"/>
-    <mergeCell ref="X7:AA7"/>
-    <mergeCell ref="BL6:BM7"/>
-    <mergeCell ref="P6:AM6"/>
-    <mergeCell ref="AN6:AR6"/>
-    <mergeCell ref="AS6:AV6"/>
-    <mergeCell ref="AW6:AZ6"/>
-    <mergeCell ref="BA6:BD6"/>
-    <mergeCell ref="BE6:BG6"/>
-    <mergeCell ref="BK7:BK8"/>
-    <mergeCell ref="AR7:AR8"/>
-    <mergeCell ref="AS7:AS8"/>
-    <mergeCell ref="AT7:AU8"/>
-    <mergeCell ref="AV7:AV8"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="AC8:AD8"/>
-    <mergeCell ref="AG8:AH8"/>
-    <mergeCell ref="P7:S7"/>
-    <mergeCell ref="T7:W7"/>
-    <mergeCell ref="BE7:BG7"/>
-    <mergeCell ref="BI7:BI8"/>
-    <mergeCell ref="BJ7:BJ8"/>
-    <mergeCell ref="AW7:AW8"/>
-    <mergeCell ref="AB7:AE7"/>
-    <mergeCell ref="AF7:AI7"/>
-    <mergeCell ref="AJ7:AM7"/>
-    <mergeCell ref="AN7:AN8"/>
-    <mergeCell ref="AO7:AP8"/>
-    <mergeCell ref="BH6:BH8"/>
-    <mergeCell ref="BI6:BK6"/>
-    <mergeCell ref="BA7:BA8"/>
-    <mergeCell ref="BB7:BB8"/>
-    <mergeCell ref="BC7:BC8"/>
-    <mergeCell ref="BD7:BD8"/>
-    <mergeCell ref="AQ7:AQ8"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
add 4 form report
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/summaryReportForm1.xlsx
+++ b/src/main/resources/templates/summaryReportForm1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1AE005B-2035-4100-BBF6-1787ED9117FD}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1E239BA-AC87-4BFB-95C0-96FFC2504A54}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="193">
   <si>
     <t>Оперативная информация</t>
   </si>
@@ -572,6 +572,33 @@
   </si>
   <si>
     <t>Кр.т. гибель озимых, га</t>
+  </si>
+  <si>
+    <t>Лен, га</t>
+  </si>
+  <si>
+    <t>$dist_value660</t>
+  </si>
+  <si>
+    <t>$dist_value658</t>
+  </si>
+  <si>
+    <t>$dist_value659</t>
+  </si>
+  <si>
+    <t>$prod_value660</t>
+  </si>
+  <si>
+    <t>$prod_value658</t>
+  </si>
+  <si>
+    <t>$prod_value659</t>
+  </si>
+  <si>
+    <t>$prod_value661</t>
+  </si>
+  <si>
+    <t>$dist_pct_value659_value660</t>
   </si>
 </sst>
 </file>
@@ -648,7 +675,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -919,36 +946,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -967,7 +964,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1005,19 +1002,16 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1038,95 +1032,107 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1408,32 +1414,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BM11"/>
+  <dimension ref="A1:BQ11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="65" width="10.7109375" customWidth="1"/>
+    <col min="3" max="69" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:69" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
-      <c r="N1" s="31"/>
-      <c r="O1" s="31"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33"/>
       <c r="P1" s="3"/>
       <c r="Q1" s="3"/>
       <c r="R1" s="3"/>
@@ -1484,25 +1490,29 @@
       <c r="BK1" s="2"/>
       <c r="BL1" s="2"/>
       <c r="BM1" s="2"/>
+      <c r="BN1" s="2"/>
+      <c r="BO1" s="2"/>
+      <c r="BP1" s="2"/>
+      <c r="BQ1" s="2"/>
     </row>
-    <row r="2" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:69" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
+      <c r="O2" s="33"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
@@ -1553,8 +1563,12 @@
       <c r="BK2" s="2"/>
       <c r="BL2" s="2"/>
       <c r="BM2" s="2"/>
+      <c r="BN2" s="2"/>
+      <c r="BO2" s="2"/>
+      <c r="BP2" s="2"/>
+      <c r="BQ2" s="2"/>
     </row>
-    <row r="3" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:69" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1624,8 +1638,12 @@
       <c r="BK3" s="2"/>
       <c r="BL3" s="2"/>
       <c r="BM3" s="2"/>
+      <c r="BN3" s="2"/>
+      <c r="BO3" s="2"/>
+      <c r="BP3" s="2"/>
+      <c r="BQ3" s="2"/>
     </row>
-    <row r="4" spans="1:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:69" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -1691,8 +1709,12 @@
       <c r="BK4" s="2"/>
       <c r="BL4" s="2"/>
       <c r="BM4" s="2"/>
+      <c r="BN4" s="2"/>
+      <c r="BO4" s="2"/>
+      <c r="BP4" s="2"/>
+      <c r="BQ4" s="2"/>
     </row>
-    <row r="5" spans="1:65" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:69" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -1720,10 +1742,10 @@
       <c r="Y5" s="4"/>
       <c r="Z5" s="4"/>
       <c r="AA5" s="4"/>
-      <c r="AB5" s="5"/>
-      <c r="AC5" s="5"/>
-      <c r="AD5" s="5"/>
-      <c r="AE5" s="5"/>
+      <c r="AB5" s="4"/>
+      <c r="AC5" s="4"/>
+      <c r="AD5" s="4"/>
+      <c r="AE5" s="4"/>
       <c r="AF5" s="5"/>
       <c r="AG5" s="5"/>
       <c r="AH5" s="5"/>
@@ -1741,271 +1763,285 @@
       <c r="AT5" s="5"/>
       <c r="AU5" s="5"/>
       <c r="AV5" s="5"/>
-      <c r="AW5" s="4"/>
-      <c r="AX5" s="4"/>
-      <c r="AY5" s="4"/>
-      <c r="AZ5" s="4"/>
+      <c r="AW5" s="5"/>
+      <c r="AX5" s="5"/>
+      <c r="AY5" s="5"/>
+      <c r="AZ5" s="5"/>
       <c r="BA5" s="4"/>
       <c r="BB5" s="4"/>
       <c r="BC5" s="4"/>
-      <c r="BD5" s="5"/>
-      <c r="BE5" s="5"/>
-      <c r="BF5" s="5"/>
-      <c r="BG5" s="6"/>
-      <c r="BH5" s="6"/>
-      <c r="BI5" s="2"/>
-      <c r="BJ5" s="2"/>
-      <c r="BK5" s="2"/>
-      <c r="BL5" s="2"/>
+      <c r="BD5" s="4"/>
+      <c r="BE5" s="4"/>
+      <c r="BF5" s="4"/>
+      <c r="BG5" s="4"/>
+      <c r="BH5" s="5"/>
+      <c r="BI5" s="5"/>
+      <c r="BJ5" s="5"/>
+      <c r="BK5" s="6"/>
+      <c r="BL5" s="6"/>
       <c r="BM5" s="2"/>
+      <c r="BN5" s="2"/>
+      <c r="BO5" s="2"/>
+      <c r="BP5" s="2"/>
+      <c r="BQ5" s="2"/>
     </row>
-    <row r="6" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="32" t="s">
+    <row r="6" spans="1:69" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="38" t="s">
+      <c r="C6" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="42" t="s">
+      <c r="F6" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="42"/>
-      <c r="H6" s="42"/>
-      <c r="I6" s="42"/>
-      <c r="J6" s="42"/>
-      <c r="K6" s="35" t="s">
+      <c r="G6" s="44"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="44"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="37" t="s">
         <v>183</v>
       </c>
-      <c r="L6" s="32" t="s">
+      <c r="L6" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="42"/>
-      <c r="N6" s="42"/>
-      <c r="O6" s="42"/>
-      <c r="P6" s="48" t="s">
+      <c r="M6" s="44"/>
+      <c r="N6" s="44"/>
+      <c r="O6" s="44"/>
+      <c r="P6" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="Q6" s="49"/>
-      <c r="R6" s="49"/>
-      <c r="S6" s="49"/>
-      <c r="T6" s="49"/>
-      <c r="U6" s="49"/>
-      <c r="V6" s="49"/>
-      <c r="W6" s="49"/>
-      <c r="X6" s="49"/>
-      <c r="Y6" s="49"/>
-      <c r="Z6" s="49"/>
-      <c r="AA6" s="49"/>
-      <c r="AB6" s="49"/>
-      <c r="AC6" s="49"/>
-      <c r="AD6" s="49"/>
-      <c r="AE6" s="49"/>
-      <c r="AF6" s="49"/>
-      <c r="AG6" s="49"/>
-      <c r="AH6" s="49"/>
-      <c r="AI6" s="49"/>
-      <c r="AJ6" s="49"/>
-      <c r="AK6" s="49"/>
-      <c r="AL6" s="49"/>
-      <c r="AM6" s="49"/>
-      <c r="AN6" s="32" t="s">
+      <c r="Q6" s="51"/>
+      <c r="R6" s="51"/>
+      <c r="S6" s="51"/>
+      <c r="T6" s="51"/>
+      <c r="U6" s="51"/>
+      <c r="V6" s="51"/>
+      <c r="W6" s="51"/>
+      <c r="X6" s="51"/>
+      <c r="Y6" s="51"/>
+      <c r="Z6" s="51"/>
+      <c r="AA6" s="51"/>
+      <c r="AB6" s="51"/>
+      <c r="AC6" s="51"/>
+      <c r="AD6" s="51"/>
+      <c r="AE6" s="51"/>
+      <c r="AF6" s="51"/>
+      <c r="AG6" s="51"/>
+      <c r="AH6" s="51"/>
+      <c r="AI6" s="51"/>
+      <c r="AJ6" s="51"/>
+      <c r="AK6" s="51"/>
+      <c r="AL6" s="51"/>
+      <c r="AM6" s="51"/>
+      <c r="AN6" s="51"/>
+      <c r="AO6" s="51"/>
+      <c r="AP6" s="51"/>
+      <c r="AQ6" s="51"/>
+      <c r="AR6" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="AO6" s="42"/>
-      <c r="AP6" s="42"/>
-      <c r="AQ6" s="42"/>
-      <c r="AR6" s="35"/>
-      <c r="AS6" s="50" t="s">
+      <c r="AS6" s="44"/>
+      <c r="AT6" s="44"/>
+      <c r="AU6" s="44"/>
+      <c r="AV6" s="37"/>
+      <c r="AW6" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="AT6" s="42"/>
-      <c r="AU6" s="42"/>
-      <c r="AV6" s="42"/>
-      <c r="AW6" s="32" t="s">
+      <c r="AX6" s="44"/>
+      <c r="AY6" s="44"/>
+      <c r="AZ6" s="44"/>
+      <c r="BA6" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="AX6" s="42"/>
-      <c r="AY6" s="42"/>
-      <c r="AZ6" s="35"/>
-      <c r="BA6" s="51" t="s">
+      <c r="BB6" s="44"/>
+      <c r="BC6" s="44"/>
+      <c r="BD6" s="37"/>
+      <c r="BE6" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="BB6" s="51"/>
-      <c r="BC6" s="51"/>
-      <c r="BD6" s="52"/>
-      <c r="BE6" s="49" t="s">
+      <c r="BF6" s="53"/>
+      <c r="BG6" s="53"/>
+      <c r="BH6" s="54"/>
+      <c r="BI6" s="51" t="s">
         <v>15</v>
       </c>
-      <c r="BF6" s="49"/>
-      <c r="BG6" s="49"/>
-      <c r="BH6" s="32" t="s">
+      <c r="BJ6" s="51"/>
+      <c r="BK6" s="51"/>
+      <c r="BL6" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="BI6" s="32" t="s">
+      <c r="BM6" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="BJ6" s="42"/>
-      <c r="BK6" s="35"/>
-      <c r="BL6" s="42" t="s">
+      <c r="BN6" s="44"/>
+      <c r="BO6" s="37"/>
+      <c r="BP6" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="BM6" s="42"/>
+      <c r="BQ6" s="44"/>
     </row>
-    <row r="7" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="33"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="39"/>
-      <c r="D7" s="41"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30" t="s">
+    <row r="7" spans="1:69" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="35"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="43" t="s">
+      <c r="G7" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="H7" s="43" t="s">
+      <c r="H7" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="30" t="s">
+      <c r="I7" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="J7" s="30" t="s">
+      <c r="J7" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="36"/>
-      <c r="L7" s="33"/>
-      <c r="M7" s="30"/>
-      <c r="N7" s="30"/>
-      <c r="O7" s="30"/>
-      <c r="P7" s="30" t="s">
+      <c r="K7" s="38"/>
+      <c r="L7" s="35"/>
+      <c r="M7" s="32"/>
+      <c r="N7" s="32"/>
+      <c r="O7" s="32"/>
+      <c r="P7" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="Q7" s="30"/>
-      <c r="R7" s="30"/>
-      <c r="S7" s="30"/>
-      <c r="T7" s="30" t="s">
+      <c r="Q7" s="32"/>
+      <c r="R7" s="32"/>
+      <c r="S7" s="32"/>
+      <c r="T7" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="U7" s="30"/>
-      <c r="V7" s="30"/>
-      <c r="W7" s="30"/>
-      <c r="X7" s="45" t="s">
+      <c r="U7" s="32"/>
+      <c r="V7" s="32"/>
+      <c r="W7" s="32"/>
+      <c r="X7" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="Y7" s="47"/>
-      <c r="Z7" s="47"/>
-      <c r="AA7" s="46"/>
-      <c r="AB7" s="30" t="s">
+      <c r="Y7" s="49"/>
+      <c r="Z7" s="49"/>
+      <c r="AA7" s="48"/>
+      <c r="AB7" s="32" t="s">
+        <v>184</v>
+      </c>
+      <c r="AC7" s="32"/>
+      <c r="AD7" s="32"/>
+      <c r="AE7" s="32"/>
+      <c r="AF7" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="AC7" s="30"/>
-      <c r="AD7" s="30"/>
-      <c r="AE7" s="30"/>
-      <c r="AF7" s="30" t="s">
+      <c r="AG7" s="32"/>
+      <c r="AH7" s="32"/>
+      <c r="AI7" s="32"/>
+      <c r="AJ7" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="AG7" s="30"/>
-      <c r="AH7" s="30"/>
-      <c r="AI7" s="30"/>
-      <c r="AJ7" s="47" t="s">
+      <c r="AK7" s="32"/>
+      <c r="AL7" s="32"/>
+      <c r="AM7" s="32"/>
+      <c r="AN7" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="AK7" s="47"/>
-      <c r="AL7" s="47"/>
-      <c r="AM7" s="47"/>
-      <c r="AN7" s="33" t="s">
+      <c r="AO7" s="49"/>
+      <c r="AP7" s="49"/>
+      <c r="AQ7" s="49"/>
+      <c r="AR7" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="AO7" s="30" t="s">
+      <c r="AS7" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="AP7" s="30"/>
-      <c r="AQ7" s="30"/>
-      <c r="AR7" s="36" t="s">
+      <c r="AT7" s="32"/>
+      <c r="AU7" s="32"/>
+      <c r="AV7" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="AS7" s="46" t="s">
+      <c r="AW7" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="AT7" s="30" t="s">
+      <c r="AX7" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="AU7" s="30"/>
-      <c r="AV7" s="30"/>
-      <c r="AW7" s="33" t="s">
+      <c r="AY7" s="32"/>
+      <c r="AZ7" s="32"/>
+      <c r="BA7" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="AX7" s="30" t="s">
+      <c r="BB7" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="AY7" s="30"/>
-      <c r="AZ7" s="36"/>
-      <c r="BA7" s="30" t="s">
+      <c r="BC7" s="32"/>
+      <c r="BD7" s="38"/>
+      <c r="BE7" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="BB7" s="30" t="s">
+      <c r="BF7" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="BC7" s="54" t="s">
+      <c r="BG7" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="BD7" s="55" t="s">
+      <c r="BH7" s="57" t="s">
         <v>36</v>
       </c>
-      <c r="BE7" s="53" t="s">
+      <c r="BI7" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="BF7" s="53"/>
-      <c r="BG7" s="53"/>
-      <c r="BH7" s="33"/>
-      <c r="BI7" s="33" t="s">
+      <c r="BJ7" s="55"/>
+      <c r="BK7" s="55"/>
+      <c r="BL7" s="35"/>
+      <c r="BM7" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="BJ7" s="30" t="s">
+      <c r="BN7" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="BK7" s="36"/>
-      <c r="BL7" s="30"/>
-      <c r="BM7" s="30"/>
+      <c r="BO7" s="38"/>
+      <c r="BP7" s="32"/>
+      <c r="BQ7" s="32"/>
     </row>
-    <row r="8" spans="1:65" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="33"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="39"/>
+    <row r="8" spans="1:69" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="35"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="41"/>
       <c r="D8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="44"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
-      <c r="K8" s="36"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="46"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="32"/>
+      <c r="K8" s="38"/>
       <c r="L8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M8" s="30" t="s">
+      <c r="M8" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="N8" s="30"/>
+      <c r="N8" s="32"/>
       <c r="O8" s="8"/>
       <c r="P8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="Q8" s="30" t="s">
+      <c r="Q8" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="R8" s="30"/>
+      <c r="R8" s="32"/>
       <c r="S8" s="8"/>
       <c r="T8" s="8" t="s">
         <v>19</v>
@@ -2022,80 +2058,88 @@
       <c r="X8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="Y8" s="45" t="s">
+      <c r="Y8" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="Z8" s="46"/>
+      <c r="Z8" s="48"/>
       <c r="AA8" s="8"/>
-      <c r="AB8" s="8" t="s">
+      <c r="AB8" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="AC8" s="30" t="s">
+      <c r="AC8" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="AD8" s="30"/>
-      <c r="AE8" s="8"/>
+      <c r="AD8" s="32"/>
+      <c r="AE8" s="28"/>
       <c r="AF8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="AG8" s="30" t="s">
+      <c r="AG8" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="AH8" s="30"/>
+      <c r="AH8" s="32"/>
       <c r="AI8" s="8"/>
       <c r="AJ8" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="AK8" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="AL8" s="32"/>
+      <c r="AM8" s="8"/>
+      <c r="AN8" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="AK8" s="8" t="s">
+      <c r="AO8" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="AL8" s="8" t="s">
+      <c r="AP8" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="AM8" s="9" t="s">
+      <c r="AQ8" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="AN8" s="33"/>
-      <c r="AO8" s="30"/>
-      <c r="AP8" s="30"/>
-      <c r="AQ8" s="30"/>
-      <c r="AR8" s="36"/>
-      <c r="AS8" s="46"/>
-      <c r="AT8" s="30"/>
-      <c r="AU8" s="30"/>
-      <c r="AV8" s="30"/>
-      <c r="AW8" s="33"/>
-      <c r="AX8" s="30"/>
-      <c r="AY8" s="30"/>
-      <c r="AZ8" s="36"/>
-      <c r="BA8" s="30"/>
-      <c r="BB8" s="30"/>
-      <c r="BC8" s="54"/>
-      <c r="BD8" s="55"/>
-      <c r="BE8" s="8" t="s">
+      <c r="AR8" s="35"/>
+      <c r="AS8" s="32"/>
+      <c r="AT8" s="32"/>
+      <c r="AU8" s="32"/>
+      <c r="AV8" s="38"/>
+      <c r="AW8" s="48"/>
+      <c r="AX8" s="32"/>
+      <c r="AY8" s="32"/>
+      <c r="AZ8" s="32"/>
+      <c r="BA8" s="35"/>
+      <c r="BB8" s="32"/>
+      <c r="BC8" s="32"/>
+      <c r="BD8" s="38"/>
+      <c r="BE8" s="32"/>
+      <c r="BF8" s="32"/>
+      <c r="BG8" s="56"/>
+      <c r="BH8" s="57"/>
+      <c r="BI8" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="BF8" s="8" t="s">
+      <c r="BJ8" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="BG8" s="8" t="s">
+      <c r="BK8" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="BH8" s="33"/>
-      <c r="BI8" s="33"/>
-      <c r="BJ8" s="30"/>
-      <c r="BK8" s="36"/>
-      <c r="BL8" s="8" t="s">
+      <c r="BL8" s="35"/>
+      <c r="BM8" s="35"/>
+      <c r="BN8" s="32"/>
+      <c r="BO8" s="38"/>
+      <c r="BP8" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="BM8" s="8" t="s">
+      <c r="BQ8" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:65" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="34"/>
-      <c r="B9" s="37"/>
-      <c r="C9" s="39"/>
+    <row r="9" spans="1:69" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="36"/>
+      <c r="B9" s="39"/>
+      <c r="C9" s="41"/>
       <c r="D9" s="10" t="s">
         <v>52</v>
       </c>
@@ -2168,16 +2212,16 @@
       <c r="AA9" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="AB9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="AC9" s="11" t="s">
+      <c r="AB9" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="AC9" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="AD9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE9" s="11" t="s">
+      <c r="AD9" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="AE9" s="29" t="s">
         <v>51</v>
       </c>
       <c r="AF9" s="11" t="s">
@@ -2196,42 +2240,42 @@
         <v>52</v>
       </c>
       <c r="AK9" s="11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="AL9" s="11" t="s">
         <v>52</v>
       </c>
       <c r="AM9" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AN9" s="11" t="s">
         <v>52</v>
       </c>
       <c r="AO9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AP9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AQ9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AR9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AS9" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="AP9" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="AQ9" s="11" t="s">
+      <c r="AT9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AU9" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="AR9" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="AS9" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="AT9" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="AU9" s="11" t="s">
-        <v>52</v>
-      </c>
       <c r="AV9" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="AW9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="AW9" s="12" t="s">
         <v>52</v>
       </c>
       <c r="AX9" s="11" t="s">
@@ -2246,14 +2290,14 @@
       <c r="BA9" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="BB9" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="BC9" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="BD9" s="10" t="s">
-        <v>52</v>
+      <c r="BB9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="BC9" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="BD9" s="12" t="s">
+        <v>51</v>
       </c>
       <c r="BE9" s="10" t="s">
         <v>52</v>
@@ -2273,21 +2317,33 @@
       <c r="BJ9" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="BK9" s="12" t="s">
+      <c r="BK9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BL9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BM9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BN9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BO9" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="BL9" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="BM9" s="10" t="s">
+      <c r="BP9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="BQ9" s="10" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:65" s="20" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="28" t="s">
+    <row r="10" spans="1:69" s="19" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="26"/>
+      <c r="B10" s="25"/>
       <c r="C10" s="15" t="s">
         <v>54</v>
       </c>
@@ -2360,360 +2416,386 @@
       <c r="Z10" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="AA10" s="17" t="s">
+      <c r="AA10" s="30" t="s">
         <v>110</v>
       </c>
       <c r="AB10" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="AC10" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="AD10" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="AE10" s="17" t="s">
+        <v>192</v>
+      </c>
+      <c r="AF10" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="AC10" s="18" t="s">
+      <c r="AG10" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="AD10" s="15" t="s">
+      <c r="AH10" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="AE10" s="17" t="s">
+      <c r="AI10" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="AF10" s="15" t="s">
+      <c r="AJ10" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="AG10" s="15" t="s">
+      <c r="AK10" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="AH10" s="15" t="s">
+      <c r="AL10" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="AI10" s="17" t="s">
+      <c r="AM10" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="AJ10" s="15" t="s">
+      <c r="AN10" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="AK10" s="15" t="s">
+      <c r="AO10" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="AL10" s="15" t="s">
+      <c r="AP10" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="AM10" s="15" t="s">
+      <c r="AQ10" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="AN10" s="15" t="s">
+      <c r="AR10" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="AO10" s="15" t="s">
+      <c r="AS10" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="AP10" s="15" t="s">
+      <c r="AT10" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="AQ10" s="16" t="s">
+      <c r="AU10" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="AR10" s="15" t="s">
+      <c r="AV10" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="AS10" s="15" t="s">
+      <c r="AW10" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="AT10" s="15" t="s">
+      <c r="AX10" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="AU10" s="15" t="s">
+      <c r="AY10" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="AV10" s="16" t="s">
+      <c r="AZ10" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="AW10" s="15" t="s">
+      <c r="BA10" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="AX10" s="15" t="s">
+      <c r="BB10" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="AY10" s="15" t="s">
+      <c r="BC10" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="AZ10" s="17" t="s">
+      <c r="BD10" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="BA10" s="15" t="s">
+      <c r="BE10" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="BB10" s="15" t="s">
+      <c r="BF10" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="BC10" s="15" t="s">
+      <c r="BG10" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="BD10" s="15" t="s">
+      <c r="BH10" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="BE10" s="15" t="s">
+      <c r="BI10" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="BF10" s="15" t="s">
+      <c r="BJ10" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="BG10" s="15" t="s">
+      <c r="BK10" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="BH10" s="15" t="s">
+      <c r="BL10" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="BI10" s="15" t="s">
+      <c r="BM10" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="BJ10" s="15" t="s">
+      <c r="BN10" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="BK10" s="17" t="s">
+      <c r="BO10" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="BL10" s="15" t="s">
+      <c r="BP10" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="BM10" s="19" t="s">
+      <c r="BQ10" s="15" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="11" spans="1:65" s="25" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="29" t="s">
+    <row r="11" spans="1:69" s="24" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="27" t="s">
         <v>116</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="D11" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="E11" s="21" t="s">
+      <c r="E11" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="G11" s="21" t="s">
+      <c r="G11" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="H11" s="21" t="s">
+      <c r="H11" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="I11" s="21" t="s">
+      <c r="I11" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="J11" s="21" t="s">
+      <c r="J11" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="K11" s="21" t="s">
+      <c r="K11" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="L11" s="21" t="s">
+      <c r="L11" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="M11" s="21" t="s">
+      <c r="M11" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="N11" s="21" t="s">
+      <c r="N11" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="O11" s="22" t="s">
+      <c r="O11" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="P11" s="21" t="s">
+      <c r="P11" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="Q11" s="21" t="s">
+      <c r="Q11" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="R11" s="21" t="s">
+      <c r="R11" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="S11" s="23" t="s">
+      <c r="S11" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="T11" s="21" t="s">
+      <c r="T11" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="U11" s="21" t="s">
+      <c r="U11" s="20" t="s">
         <v>136</v>
       </c>
-      <c r="V11" s="21" t="s">
+      <c r="V11" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="W11" s="21" t="s">
+      <c r="W11" s="20" t="s">
         <v>138</v>
       </c>
-      <c r="X11" s="21" t="s">
+      <c r="X11" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="Y11" s="21" t="s">
+      <c r="Y11" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="Z11" s="21" t="s">
+      <c r="Z11" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="AA11" s="23" t="s">
+      <c r="AA11" s="31" t="s">
         <v>142</v>
       </c>
-      <c r="AB11" s="21" t="s">
+      <c r="AB11" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="AC11" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="AD11" s="20" t="s">
+        <v>190</v>
+      </c>
+      <c r="AE11" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="AF11" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="AC11" s="24" t="s">
+      <c r="AG11" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="AD11" s="21" t="s">
+      <c r="AH11" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="AE11" s="23" t="s">
+      <c r="AI11" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="AF11" s="21" t="s">
+      <c r="AJ11" s="20" t="s">
         <v>147</v>
       </c>
-      <c r="AG11" s="21" t="s">
+      <c r="AK11" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="AH11" s="21" t="s">
+      <c r="AL11" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="AI11" s="23" t="s">
+      <c r="AM11" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="AJ11" s="21" t="s">
+      <c r="AN11" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="AK11" s="21" t="s">
+      <c r="AO11" s="20" t="s">
         <v>152</v>
       </c>
-      <c r="AL11" s="21" t="s">
+      <c r="AP11" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="AM11" s="21" t="s">
+      <c r="AQ11" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="AN11" s="21" t="s">
+      <c r="AR11" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="AO11" s="21" t="s">
+      <c r="AS11" s="20" t="s">
         <v>156</v>
       </c>
-      <c r="AP11" s="21" t="s">
+      <c r="AT11" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="AQ11" s="22" t="s">
+      <c r="AU11" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="AR11" s="21" t="s">
+      <c r="AV11" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="AS11" s="21" t="s">
+      <c r="AW11" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="AT11" s="21" t="s">
+      <c r="AX11" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="AU11" s="21" t="s">
+      <c r="AY11" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="AV11" s="22" t="s">
+      <c r="AZ11" s="21" t="s">
         <v>163</v>
       </c>
-      <c r="AW11" s="21" t="s">
+      <c r="BA11" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="AX11" s="21" t="s">
+      <c r="BB11" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="AY11" s="21" t="s">
+      <c r="BC11" s="20" t="s">
         <v>166</v>
       </c>
-      <c r="AZ11" s="23" t="s">
+      <c r="BD11" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="BA11" s="21" t="s">
+      <c r="BE11" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="BB11" s="21" t="s">
+      <c r="BF11" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="BC11" s="21" t="s">
+      <c r="BG11" s="20" t="s">
         <v>170</v>
       </c>
-      <c r="BD11" s="21" t="s">
+      <c r="BH11" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="BE11" s="21" t="s">
+      <c r="BI11" s="20" t="s">
         <v>172</v>
       </c>
-      <c r="BF11" s="21" t="s">
+      <c r="BJ11" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="BG11" s="21" t="s">
+      <c r="BK11" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="BH11" s="21" t="s">
+      <c r="BL11" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="BI11" s="21" t="s">
+      <c r="BM11" s="20" t="s">
         <v>176</v>
       </c>
-      <c r="BJ11" s="21" t="s">
+      <c r="BN11" s="20" t="s">
         <v>177</v>
       </c>
-      <c r="BK11" s="23" t="s">
+      <c r="BO11" s="22" t="s">
         <v>178</v>
       </c>
-      <c r="BL11" s="21" t="s">
+      <c r="BP11" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="BM11" s="21" t="s">
+      <c r="BQ11" s="20" t="s">
         <v>180</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="53">
-    <mergeCell ref="BE7:BG7"/>
-    <mergeCell ref="BI7:BI8"/>
-    <mergeCell ref="BJ7:BJ8"/>
-    <mergeCell ref="AW7:AW8"/>
-    <mergeCell ref="AB7:AE7"/>
+  <mergeCells count="55">
+    <mergeCell ref="BI7:BK7"/>
+    <mergeCell ref="BM7:BM8"/>
+    <mergeCell ref="BN7:BN8"/>
+    <mergeCell ref="BA7:BA8"/>
     <mergeCell ref="AF7:AI7"/>
     <mergeCell ref="AJ7:AM7"/>
-    <mergeCell ref="AN7:AN8"/>
-    <mergeCell ref="AO7:AP8"/>
-    <mergeCell ref="BH6:BH8"/>
-    <mergeCell ref="BI6:BK6"/>
-    <mergeCell ref="BA7:BA8"/>
-    <mergeCell ref="BB7:BB8"/>
-    <mergeCell ref="BC7:BC8"/>
-    <mergeCell ref="BD7:BD8"/>
-    <mergeCell ref="AQ7:AQ8"/>
+    <mergeCell ref="AN7:AQ7"/>
+    <mergeCell ref="AR7:AR8"/>
+    <mergeCell ref="AS7:AT8"/>
+    <mergeCell ref="BL6:BL8"/>
+    <mergeCell ref="BM6:BO6"/>
+    <mergeCell ref="BE7:BE8"/>
+    <mergeCell ref="BF7:BF8"/>
+    <mergeCell ref="BG7:BG8"/>
+    <mergeCell ref="BH7:BH8"/>
+    <mergeCell ref="AU7:AU8"/>
     <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="AC8:AD8"/>
     <mergeCell ref="AG8:AH8"/>
+    <mergeCell ref="AK8:AL8"/>
     <mergeCell ref="P7:S7"/>
     <mergeCell ref="T7:W7"/>
+    <mergeCell ref="AB7:AE7"/>
+    <mergeCell ref="AC8:AD8"/>
+    <mergeCell ref="BB7:BC8"/>
+    <mergeCell ref="BD7:BD8"/>
+    <mergeCell ref="Y8:Z8"/>
+    <mergeCell ref="X7:AA7"/>
+    <mergeCell ref="BP6:BQ7"/>
+    <mergeCell ref="P6:AQ6"/>
+    <mergeCell ref="AR6:AV6"/>
+    <mergeCell ref="AW6:AZ6"/>
+    <mergeCell ref="BA6:BD6"/>
+    <mergeCell ref="BE6:BH6"/>
+    <mergeCell ref="BI6:BK6"/>
+    <mergeCell ref="BO7:BO8"/>
+    <mergeCell ref="AV7:AV8"/>
+    <mergeCell ref="AW7:AW8"/>
     <mergeCell ref="AX7:AY8"/>
     <mergeCell ref="AZ7:AZ8"/>
-    <mergeCell ref="Y8:Z8"/>
-    <mergeCell ref="X7:AA7"/>
-    <mergeCell ref="BL6:BM7"/>
-    <mergeCell ref="P6:AM6"/>
-    <mergeCell ref="AN6:AR6"/>
-    <mergeCell ref="AS6:AV6"/>
-    <mergeCell ref="AW6:AZ6"/>
-    <mergeCell ref="BA6:BD6"/>
-    <mergeCell ref="BE6:BG6"/>
-    <mergeCell ref="BK7:BK8"/>
-    <mergeCell ref="AR7:AR8"/>
-    <mergeCell ref="AS7:AS8"/>
-    <mergeCell ref="AT7:AU8"/>
-    <mergeCell ref="AV7:AV8"/>
     <mergeCell ref="M8:N8"/>
     <mergeCell ref="B1:O1"/>
     <mergeCell ref="B2:O2"/>

</xml_diff>

<commit_message>
fix template's values quality
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/summaryReportForm1.xlsx
+++ b/src/main/resources/templates/summaryReportForm1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{132C858E-9A81-49F6-B9E0-4505917628EE}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BCCF2B4-B564-4753-AF38-7FE8D43B770E}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -605,6 +605,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -964,7 +967,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1002,117 +1005,42 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1128,11 +1056,74 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1417,29 +1408,29 @@
   <dimension ref="A1:BQ11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="45.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
     <col min="3" max="69" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
-      <c r="B1" s="50" t="s">
+      <c r="B1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="50"/>
-      <c r="M1" s="50"/>
-      <c r="N1" s="50"/>
-      <c r="O1" s="50"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
       <c r="P1" s="3"/>
       <c r="Q1" s="3"/>
       <c r="R1" s="3"/>
@@ -1497,22 +1488,22 @@
     </row>
     <row r="2" spans="1:69" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="50" t="s">
+      <c r="B2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-      <c r="K2" s="50"/>
-      <c r="L2" s="50"/>
-      <c r="M2" s="50"/>
-      <c r="N2" s="50"/>
-      <c r="O2" s="50"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
@@ -1786,262 +1777,262 @@
       <c r="BQ5" s="2"/>
     </row>
     <row r="6" spans="1:69" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="53" t="s">
+      <c r="C6" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="55" t="s">
+      <c r="D6" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="38" t="s">
+      <c r="E6" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="38" t="s">
+      <c r="F6" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="38"/>
-      <c r="H6" s="38"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="39" t="s">
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="25" t="s">
         <v>181</v>
       </c>
-      <c r="L6" s="37" t="s">
+      <c r="L6" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="38"/>
-      <c r="N6" s="38"/>
-      <c r="O6" s="38"/>
-      <c r="P6" s="45" t="s">
+      <c r="M6" s="32"/>
+      <c r="N6" s="32"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="Q6" s="46"/>
-      <c r="R6" s="46"/>
-      <c r="S6" s="46"/>
-      <c r="T6" s="46"/>
-      <c r="U6" s="46"/>
-      <c r="V6" s="46"/>
-      <c r="W6" s="46"/>
-      <c r="X6" s="46"/>
-      <c r="Y6" s="46"/>
-      <c r="Z6" s="46"/>
-      <c r="AA6" s="46"/>
-      <c r="AB6" s="46"/>
-      <c r="AC6" s="46"/>
-      <c r="AD6" s="46"/>
-      <c r="AE6" s="46"/>
-      <c r="AF6" s="46"/>
-      <c r="AG6" s="46"/>
-      <c r="AH6" s="46"/>
-      <c r="AI6" s="46"/>
-      <c r="AJ6" s="46"/>
-      <c r="AK6" s="46"/>
-      <c r="AL6" s="46"/>
-      <c r="AM6" s="46"/>
-      <c r="AN6" s="46"/>
-      <c r="AO6" s="46"/>
-      <c r="AP6" s="46"/>
-      <c r="AQ6" s="46"/>
-      <c r="AR6" s="37" t="s">
+      <c r="Q6" s="39"/>
+      <c r="R6" s="39"/>
+      <c r="S6" s="39"/>
+      <c r="T6" s="39"/>
+      <c r="U6" s="39"/>
+      <c r="V6" s="39"/>
+      <c r="W6" s="39"/>
+      <c r="X6" s="39"/>
+      <c r="Y6" s="39"/>
+      <c r="Z6" s="39"/>
+      <c r="AA6" s="39"/>
+      <c r="AB6" s="39"/>
+      <c r="AC6" s="39"/>
+      <c r="AD6" s="39"/>
+      <c r="AE6" s="39"/>
+      <c r="AF6" s="39"/>
+      <c r="AG6" s="39"/>
+      <c r="AH6" s="39"/>
+      <c r="AI6" s="39"/>
+      <c r="AJ6" s="39"/>
+      <c r="AK6" s="39"/>
+      <c r="AL6" s="39"/>
+      <c r="AM6" s="39"/>
+      <c r="AN6" s="39"/>
+      <c r="AO6" s="39"/>
+      <c r="AP6" s="39"/>
+      <c r="AQ6" s="39"/>
+      <c r="AR6" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="AS6" s="38"/>
-      <c r="AT6" s="38"/>
-      <c r="AU6" s="38"/>
-      <c r="AV6" s="39"/>
-      <c r="AW6" s="47" t="s">
+      <c r="AS6" s="32"/>
+      <c r="AT6" s="32"/>
+      <c r="AU6" s="32"/>
+      <c r="AV6" s="25"/>
+      <c r="AW6" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="AX6" s="38"/>
-      <c r="AY6" s="38"/>
-      <c r="AZ6" s="38"/>
-      <c r="BA6" s="37" t="s">
+      <c r="AX6" s="32"/>
+      <c r="AY6" s="32"/>
+      <c r="AZ6" s="32"/>
+      <c r="BA6" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="BB6" s="38"/>
-      <c r="BC6" s="38"/>
-      <c r="BD6" s="39"/>
-      <c r="BE6" s="48" t="s">
+      <c r="BB6" s="32"/>
+      <c r="BC6" s="32"/>
+      <c r="BD6" s="25"/>
+      <c r="BE6" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="BF6" s="48"/>
-      <c r="BG6" s="48"/>
-      <c r="BH6" s="49"/>
-      <c r="BI6" s="46" t="s">
+      <c r="BF6" s="41"/>
+      <c r="BG6" s="41"/>
+      <c r="BH6" s="42"/>
+      <c r="BI6" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="BJ6" s="46"/>
-      <c r="BK6" s="46"/>
-      <c r="BL6" s="37" t="s">
+      <c r="BJ6" s="39"/>
+      <c r="BK6" s="39"/>
+      <c r="BL6" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="BM6" s="37" t="s">
+      <c r="BM6" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="BN6" s="38"/>
-      <c r="BO6" s="39"/>
-      <c r="BP6" s="38" t="s">
+      <c r="BN6" s="32"/>
+      <c r="BO6" s="25"/>
+      <c r="BP6" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="BQ6" s="38"/>
+      <c r="BQ6" s="32"/>
     </row>
     <row r="7" spans="1:69" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="34"/>
-      <c r="B7" s="42"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="56"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35" t="s">
+      <c r="A7" s="23"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="57" t="s">
+      <c r="G7" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="H7" s="57" t="s">
+      <c r="H7" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="35" t="s">
+      <c r="I7" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="J7" s="35" t="s">
+      <c r="J7" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="42"/>
-      <c r="L7" s="34"/>
-      <c r="M7" s="35"/>
-      <c r="N7" s="35"/>
-      <c r="O7" s="35"/>
-      <c r="P7" s="35" t="s">
+      <c r="K7" s="26"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="20"/>
+      <c r="N7" s="20"/>
+      <c r="O7" s="20"/>
+      <c r="P7" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="Q7" s="35"/>
-      <c r="R7" s="35"/>
-      <c r="S7" s="35"/>
-      <c r="T7" s="35" t="s">
+      <c r="Q7" s="20"/>
+      <c r="R7" s="20"/>
+      <c r="S7" s="20"/>
+      <c r="T7" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="U7" s="35"/>
-      <c r="V7" s="35"/>
-      <c r="W7" s="35"/>
-      <c r="X7" s="43" t="s">
+      <c r="U7" s="20"/>
+      <c r="V7" s="20"/>
+      <c r="W7" s="20"/>
+      <c r="X7" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="Y7" s="36"/>
-      <c r="Z7" s="36"/>
-      <c r="AA7" s="44"/>
-      <c r="AB7" s="35" t="s">
+      <c r="Y7" s="37"/>
+      <c r="Z7" s="37"/>
+      <c r="AA7" s="36"/>
+      <c r="AB7" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="AC7" s="35"/>
-      <c r="AD7" s="35"/>
-      <c r="AE7" s="35"/>
-      <c r="AF7" s="35" t="s">
+      <c r="AC7" s="20"/>
+      <c r="AD7" s="20"/>
+      <c r="AE7" s="20"/>
+      <c r="AF7" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="AG7" s="35"/>
-      <c r="AH7" s="35"/>
-      <c r="AI7" s="35"/>
-      <c r="AJ7" s="35" t="s">
+      <c r="AG7" s="20"/>
+      <c r="AH7" s="20"/>
+      <c r="AI7" s="20"/>
+      <c r="AJ7" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="AK7" s="35"/>
-      <c r="AL7" s="35"/>
-      <c r="AM7" s="35"/>
-      <c r="AN7" s="36" t="s">
+      <c r="AK7" s="20"/>
+      <c r="AL7" s="20"/>
+      <c r="AM7" s="20"/>
+      <c r="AN7" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AO7" s="36"/>
-      <c r="AP7" s="36"/>
-      <c r="AQ7" s="36"/>
-      <c r="AR7" s="34" t="s">
+      <c r="AO7" s="37"/>
+      <c r="AP7" s="37"/>
+      <c r="AQ7" s="37"/>
+      <c r="AR7" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="AS7" s="35" t="s">
+      <c r="AS7" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="AT7" s="35"/>
-      <c r="AU7" s="35"/>
-      <c r="AV7" s="42" t="s">
+      <c r="AT7" s="20"/>
+      <c r="AU7" s="20"/>
+      <c r="AV7" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="AW7" s="44" t="s">
+      <c r="AW7" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="AX7" s="35" t="s">
+      <c r="AX7" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="AY7" s="35"/>
-      <c r="AZ7" s="35"/>
-      <c r="BA7" s="34" t="s">
+      <c r="AY7" s="20"/>
+      <c r="AZ7" s="20"/>
+      <c r="BA7" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="BB7" s="35" t="s">
+      <c r="BB7" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="BC7" s="35"/>
-      <c r="BD7" s="42"/>
-      <c r="BE7" s="35" t="s">
+      <c r="BC7" s="20"/>
+      <c r="BD7" s="26"/>
+      <c r="BE7" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="BF7" s="35" t="s">
+      <c r="BF7" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="BG7" s="40" t="s">
+      <c r="BG7" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="BH7" s="41" t="s">
+      <c r="BH7" s="45" t="s">
         <v>36</v>
       </c>
-      <c r="BI7" s="33" t="s">
+      <c r="BI7" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="BJ7" s="33"/>
-      <c r="BK7" s="33"/>
-      <c r="BL7" s="34"/>
-      <c r="BM7" s="34" t="s">
+      <c r="BJ7" s="43"/>
+      <c r="BK7" s="43"/>
+      <c r="BL7" s="23"/>
+      <c r="BM7" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="BN7" s="35" t="s">
+      <c r="BN7" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="BO7" s="42"/>
-      <c r="BP7" s="35"/>
-      <c r="BQ7" s="35"/>
+      <c r="BO7" s="26"/>
+      <c r="BP7" s="20"/>
+      <c r="BQ7" s="20"/>
     </row>
     <row r="8" spans="1:69" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="34"/>
-      <c r="B8" s="42"/>
-      <c r="C8" s="54"/>
+      <c r="A8" s="23"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="29"/>
       <c r="D8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="58"/>
-      <c r="H8" s="58"/>
-      <c r="I8" s="35"/>
-      <c r="J8" s="35"/>
-      <c r="K8" s="42"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="26"/>
       <c r="L8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M8" s="35" t="s">
+      <c r="M8" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="N8" s="35"/>
+      <c r="N8" s="20"/>
       <c r="O8" s="8"/>
       <c r="P8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="Q8" s="35" t="s">
+      <c r="Q8" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="R8" s="35"/>
+      <c r="R8" s="20"/>
       <c r="S8" s="8"/>
       <c r="T8" s="8" t="s">
         <v>19</v>
@@ -2058,34 +2049,34 @@
       <c r="X8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="Y8" s="43" t="s">
+      <c r="Y8" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="Z8" s="44"/>
+      <c r="Z8" s="36"/>
       <c r="AA8" s="8"/>
-      <c r="AB8" s="28" t="s">
+      <c r="AB8" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="AC8" s="35" t="s">
+      <c r="AC8" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="AD8" s="35"/>
-      <c r="AE8" s="28"/>
+      <c r="AD8" s="20"/>
+      <c r="AE8" s="17"/>
       <c r="AF8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="AG8" s="35" t="s">
+      <c r="AG8" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="AH8" s="35"/>
+      <c r="AH8" s="20"/>
       <c r="AI8" s="8"/>
       <c r="AJ8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="AK8" s="35" t="s">
+      <c r="AK8" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="AL8" s="35"/>
+      <c r="AL8" s="20"/>
       <c r="AM8" s="8"/>
       <c r="AN8" s="8" t="s">
         <v>42</v>
@@ -2099,23 +2090,23 @@
       <c r="AQ8" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="AR8" s="34"/>
-      <c r="AS8" s="35"/>
-      <c r="AT8" s="35"/>
-      <c r="AU8" s="35"/>
-      <c r="AV8" s="42"/>
-      <c r="AW8" s="44"/>
-      <c r="AX8" s="35"/>
-      <c r="AY8" s="35"/>
-      <c r="AZ8" s="35"/>
-      <c r="BA8" s="34"/>
-      <c r="BB8" s="35"/>
-      <c r="BC8" s="35"/>
-      <c r="BD8" s="42"/>
-      <c r="BE8" s="35"/>
-      <c r="BF8" s="35"/>
-      <c r="BG8" s="40"/>
-      <c r="BH8" s="41"/>
+      <c r="AR8" s="23"/>
+      <c r="AS8" s="20"/>
+      <c r="AT8" s="20"/>
+      <c r="AU8" s="20"/>
+      <c r="AV8" s="26"/>
+      <c r="AW8" s="36"/>
+      <c r="AX8" s="20"/>
+      <c r="AY8" s="20"/>
+      <c r="AZ8" s="20"/>
+      <c r="BA8" s="23"/>
+      <c r="BB8" s="20"/>
+      <c r="BC8" s="20"/>
+      <c r="BD8" s="26"/>
+      <c r="BE8" s="20"/>
+      <c r="BF8" s="20"/>
+      <c r="BG8" s="44"/>
+      <c r="BH8" s="45"/>
       <c r="BI8" s="8" t="s">
         <v>46</v>
       </c>
@@ -2125,10 +2116,10 @@
       <c r="BK8" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="BL8" s="34"/>
-      <c r="BM8" s="34"/>
-      <c r="BN8" s="35"/>
-      <c r="BO8" s="42"/>
+      <c r="BL8" s="23"/>
+      <c r="BM8" s="23"/>
+      <c r="BN8" s="20"/>
+      <c r="BO8" s="26"/>
       <c r="BP8" s="8" t="s">
         <v>49</v>
       </c>
@@ -2137,9 +2128,9 @@
       </c>
     </row>
     <row r="9" spans="1:69" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="51"/>
-      <c r="B9" s="52"/>
-      <c r="C9" s="54"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="29"/>
       <c r="D9" s="10" t="s">
         <v>192</v>
       </c>
@@ -2212,16 +2203,16 @@
       <c r="AA9" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="AB9" s="29" t="s">
-        <v>192</v>
-      </c>
-      <c r="AC9" s="29" t="s">
+      <c r="AB9" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="AC9" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="AD9" s="29" t="s">
-        <v>192</v>
-      </c>
-      <c r="AE9" s="29" t="s">
+      <c r="AD9" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="AE9" s="18" t="s">
         <v>51</v>
       </c>
       <c r="AF9" s="11" t="s">
@@ -2339,424 +2330,463 @@
         <v>192</v>
       </c>
     </row>
-    <row r="10" spans="1:69" s="19" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="32" t="s">
+    <row r="10" spans="1:69" s="15" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="25"/>
-      <c r="C10" s="15" t="s">
+      <c r="B10" s="52"/>
+      <c r="C10" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E10" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="G10" s="46" t="s">
         <v>57</v>
       </c>
-      <c r="H10" s="15" t="s">
+      <c r="H10" s="46" t="s">
         <v>58</v>
       </c>
-      <c r="I10" s="15" t="s">
+      <c r="I10" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="J10" s="15" t="s">
+      <c r="J10" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="K10" s="15" t="s">
+      <c r="K10" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="L10" s="15" t="s">
+      <c r="L10" s="46" t="s">
         <v>62</v>
       </c>
-      <c r="M10" s="15" t="s">
+      <c r="M10" s="46" t="s">
         <v>63</v>
       </c>
-      <c r="N10" s="15" t="s">
+      <c r="N10" s="46" t="s">
         <v>64</v>
       </c>
-      <c r="O10" s="16" t="s">
+      <c r="O10" s="46" t="s">
         <v>107</v>
       </c>
-      <c r="P10" s="15" t="s">
+      <c r="P10" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="Q10" s="15" t="s">
+      <c r="Q10" s="46" t="s">
         <v>66</v>
       </c>
-      <c r="R10" s="15" t="s">
+      <c r="R10" s="46" t="s">
         <v>67</v>
       </c>
-      <c r="S10" s="17" t="s">
+      <c r="S10" s="47" t="s">
         <v>108</v>
       </c>
-      <c r="T10" s="15" t="s">
+      <c r="T10" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="U10" s="15" t="s">
+      <c r="U10" s="46" t="s">
         <v>69</v>
       </c>
-      <c r="V10" s="15" t="s">
+      <c r="V10" s="46" t="s">
         <v>70</v>
       </c>
-      <c r="W10" s="15" t="s">
+      <c r="W10" s="46" t="s">
         <v>71</v>
       </c>
-      <c r="X10" s="15" t="s">
+      <c r="X10" s="46" t="s">
         <v>72</v>
       </c>
-      <c r="Y10" s="15" t="s">
+      <c r="Y10" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="Z10" s="15" t="s">
+      <c r="Z10" s="46" t="s">
         <v>74</v>
       </c>
-      <c r="AA10" s="30" t="s">
+      <c r="AA10" s="48" t="s">
         <v>109</v>
       </c>
-      <c r="AB10" s="15" t="s">
+      <c r="AB10" s="46" t="s">
         <v>183</v>
       </c>
-      <c r="AC10" s="18" t="s">
+      <c r="AC10" s="47" t="s">
         <v>184</v>
       </c>
-      <c r="AD10" s="15" t="s">
+      <c r="AD10" s="46" t="s">
         <v>185</v>
       </c>
-      <c r="AE10" s="17" t="s">
+      <c r="AE10" s="47" t="s">
         <v>190</v>
       </c>
-      <c r="AF10" s="15" t="s">
+      <c r="AF10" s="46" t="s">
         <v>76</v>
       </c>
-      <c r="AG10" s="18" t="s">
+      <c r="AG10" s="47" t="s">
         <v>75</v>
       </c>
-      <c r="AH10" s="15" t="s">
+      <c r="AH10" s="46" t="s">
         <v>77</v>
       </c>
-      <c r="AI10" s="17" t="s">
+      <c r="AI10" s="47" t="s">
         <v>180</v>
       </c>
-      <c r="AJ10" s="15" t="s">
+      <c r="AJ10" s="46" t="s">
         <v>78</v>
       </c>
-      <c r="AK10" s="15" t="s">
+      <c r="AK10" s="46" t="s">
         <v>79</v>
       </c>
-      <c r="AL10" s="15" t="s">
+      <c r="AL10" s="46" t="s">
         <v>80</v>
       </c>
-      <c r="AM10" s="17" t="s">
+      <c r="AM10" s="47" t="s">
         <v>110</v>
       </c>
-      <c r="AN10" s="15" t="s">
+      <c r="AN10" s="46" t="s">
         <v>81</v>
       </c>
-      <c r="AO10" s="15" t="s">
+      <c r="AO10" s="46" t="s">
         <v>82</v>
       </c>
-      <c r="AP10" s="15" t="s">
+      <c r="AP10" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="AQ10" s="15" t="s">
+      <c r="AQ10" s="46" t="s">
         <v>84</v>
       </c>
-      <c r="AR10" s="15" t="s">
+      <c r="AR10" s="46" t="s">
         <v>85</v>
       </c>
-      <c r="AS10" s="15" t="s">
+      <c r="AS10" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="AT10" s="15" t="s">
+      <c r="AT10" s="46" t="s">
         <v>87</v>
       </c>
-      <c r="AU10" s="16" t="s">
+      <c r="AU10" s="46" t="s">
         <v>111</v>
       </c>
-      <c r="AV10" s="15" t="s">
+      <c r="AV10" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="AW10" s="15" t="s">
+      <c r="AW10" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="AX10" s="15" t="s">
+      <c r="AX10" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="AY10" s="15" t="s">
+      <c r="AY10" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="AZ10" s="16" t="s">
+      <c r="AZ10" s="46" t="s">
         <v>112</v>
       </c>
-      <c r="BA10" s="15" t="s">
+      <c r="BA10" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="BB10" s="15" t="s">
+      <c r="BB10" s="46" t="s">
         <v>93</v>
       </c>
-      <c r="BC10" s="15" t="s">
+      <c r="BC10" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="BD10" s="17" t="s">
+      <c r="BD10" s="47" t="s">
         <v>113</v>
       </c>
-      <c r="BE10" s="15" t="s">
+      <c r="BE10" s="46" t="s">
         <v>95</v>
       </c>
-      <c r="BF10" s="15" t="s">
+      <c r="BF10" s="46" t="s">
         <v>96</v>
       </c>
-      <c r="BG10" s="15" t="s">
+      <c r="BG10" s="46" t="s">
         <v>97</v>
       </c>
-      <c r="BH10" s="15" t="s">
+      <c r="BH10" s="46" t="s">
         <v>98</v>
       </c>
-      <c r="BI10" s="15" t="s">
+      <c r="BI10" s="46" t="s">
         <v>99</v>
       </c>
-      <c r="BJ10" s="15" t="s">
+      <c r="BJ10" s="46" t="s">
         <v>100</v>
       </c>
-      <c r="BK10" s="15" t="s">
+      <c r="BK10" s="46" t="s">
         <v>101</v>
       </c>
-      <c r="BL10" s="15" t="s">
+      <c r="BL10" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="BM10" s="15" t="s">
+      <c r="BM10" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="BN10" s="15" t="s">
+      <c r="BN10" s="46" t="s">
         <v>104</v>
       </c>
-      <c r="BO10" s="17" t="s">
+      <c r="BO10" s="47" t="s">
         <v>114</v>
       </c>
-      <c r="BP10" s="15" t="s">
+      <c r="BP10" s="46" t="s">
         <v>105</v>
       </c>
-      <c r="BQ10" s="15" t="s">
+      <c r="BQ10" s="46" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:69" s="24" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
+    <row r="11" spans="1:69" s="16" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="53" t="s">
         <v>115</v>
       </c>
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="54" t="s">
         <v>116</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="49" t="s">
         <v>117</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="49" t="s">
         <v>118</v>
       </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="49" t="s">
         <v>119</v>
       </c>
-      <c r="F11" s="20" t="s">
+      <c r="F11" s="49" t="s">
         <v>120</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="G11" s="49" t="s">
         <v>121</v>
       </c>
-      <c r="H11" s="20" t="s">
+      <c r="H11" s="49" t="s">
         <v>122</v>
       </c>
-      <c r="I11" s="20" t="s">
+      <c r="I11" s="49" t="s">
         <v>123</v>
       </c>
-      <c r="J11" s="20" t="s">
+      <c r="J11" s="49" t="s">
         <v>124</v>
       </c>
-      <c r="K11" s="20" t="s">
+      <c r="K11" s="49" t="s">
         <v>125</v>
       </c>
-      <c r="L11" s="20" t="s">
+      <c r="L11" s="49" t="s">
         <v>126</v>
       </c>
-      <c r="M11" s="20" t="s">
+      <c r="M11" s="49" t="s">
         <v>127</v>
       </c>
-      <c r="N11" s="20" t="s">
+      <c r="N11" s="49" t="s">
         <v>128</v>
       </c>
-      <c r="O11" s="21" t="s">
+      <c r="O11" s="49" t="s">
         <v>129</v>
       </c>
-      <c r="P11" s="20" t="s">
+      <c r="P11" s="49" t="s">
         <v>130</v>
       </c>
-      <c r="Q11" s="20" t="s">
+      <c r="Q11" s="49" t="s">
         <v>131</v>
       </c>
-      <c r="R11" s="20" t="s">
+      <c r="R11" s="49" t="s">
         <v>132</v>
       </c>
-      <c r="S11" s="22" t="s">
+      <c r="S11" s="50" t="s">
         <v>133</v>
       </c>
-      <c r="T11" s="20" t="s">
+      <c r="T11" s="49" t="s">
         <v>134</v>
       </c>
-      <c r="U11" s="20" t="s">
+      <c r="U11" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="V11" s="20" t="s">
+      <c r="V11" s="49" t="s">
         <v>136</v>
       </c>
-      <c r="W11" s="20" t="s">
+      <c r="W11" s="49" t="s">
         <v>137</v>
       </c>
-      <c r="X11" s="20" t="s">
+      <c r="X11" s="49" t="s">
         <v>138</v>
       </c>
-      <c r="Y11" s="20" t="s">
+      <c r="Y11" s="49" t="s">
         <v>139</v>
       </c>
-      <c r="Z11" s="20" t="s">
+      <c r="Z11" s="49" t="s">
         <v>140</v>
       </c>
-      <c r="AA11" s="31" t="s">
+      <c r="AA11" s="51" t="s">
         <v>141</v>
       </c>
-      <c r="AB11" s="20" t="s">
+      <c r="AB11" s="49" t="s">
         <v>186</v>
       </c>
-      <c r="AC11" s="23" t="s">
+      <c r="AC11" s="50" t="s">
         <v>187</v>
       </c>
-      <c r="AD11" s="20" t="s">
+      <c r="AD11" s="49" t="s">
         <v>188</v>
       </c>
-      <c r="AE11" s="22" t="s">
+      <c r="AE11" s="50" t="s">
         <v>189</v>
       </c>
-      <c r="AF11" s="20" t="s">
+      <c r="AF11" s="49" t="s">
         <v>143</v>
       </c>
-      <c r="AG11" s="23" t="s">
+      <c r="AG11" s="50" t="s">
         <v>142</v>
       </c>
-      <c r="AH11" s="20" t="s">
+      <c r="AH11" s="49" t="s">
         <v>144</v>
       </c>
-      <c r="AI11" s="22" t="s">
+      <c r="AI11" s="50" t="s">
         <v>145</v>
       </c>
-      <c r="AJ11" s="20" t="s">
+      <c r="AJ11" s="49" t="s">
         <v>146</v>
       </c>
-      <c r="AK11" s="20" t="s">
+      <c r="AK11" s="49" t="s">
         <v>147</v>
       </c>
-      <c r="AL11" s="20" t="s">
+      <c r="AL11" s="49" t="s">
         <v>148</v>
       </c>
-      <c r="AM11" s="22" t="s">
+      <c r="AM11" s="50" t="s">
         <v>149</v>
       </c>
-      <c r="AN11" s="20" t="s">
+      <c r="AN11" s="49" t="s">
         <v>150</v>
       </c>
-      <c r="AO11" s="20" t="s">
+      <c r="AO11" s="49" t="s">
         <v>151</v>
       </c>
-      <c r="AP11" s="20" t="s">
+      <c r="AP11" s="49" t="s">
         <v>152</v>
       </c>
-      <c r="AQ11" s="20" t="s">
+      <c r="AQ11" s="49" t="s">
         <v>153</v>
       </c>
-      <c r="AR11" s="20" t="s">
+      <c r="AR11" s="49" t="s">
         <v>154</v>
       </c>
-      <c r="AS11" s="20" t="s">
+      <c r="AS11" s="49" t="s">
         <v>155</v>
       </c>
-      <c r="AT11" s="20" t="s">
+      <c r="AT11" s="49" t="s">
         <v>156</v>
       </c>
-      <c r="AU11" s="21" t="s">
+      <c r="AU11" s="49" t="s">
         <v>157</v>
       </c>
-      <c r="AV11" s="20" t="s">
+      <c r="AV11" s="49" t="s">
         <v>158</v>
       </c>
-      <c r="AW11" s="20" t="s">
+      <c r="AW11" s="49" t="s">
         <v>159</v>
       </c>
-      <c r="AX11" s="20" t="s">
+      <c r="AX11" s="49" t="s">
         <v>160</v>
       </c>
-      <c r="AY11" s="20" t="s">
+      <c r="AY11" s="49" t="s">
         <v>161</v>
       </c>
-      <c r="AZ11" s="21" t="s">
+      <c r="AZ11" s="49" t="s">
         <v>162</v>
       </c>
-      <c r="BA11" s="20" t="s">
+      <c r="BA11" s="49" t="s">
         <v>163</v>
       </c>
-      <c r="BB11" s="20" t="s">
+      <c r="BB11" s="49" t="s">
         <v>164</v>
       </c>
-      <c r="BC11" s="20" t="s">
+      <c r="BC11" s="49" t="s">
         <v>165</v>
       </c>
-      <c r="BD11" s="22" t="s">
+      <c r="BD11" s="50" t="s">
         <v>166</v>
       </c>
-      <c r="BE11" s="20" t="s">
+      <c r="BE11" s="49" t="s">
         <v>167</v>
       </c>
-      <c r="BF11" s="20" t="s">
+      <c r="BF11" s="49" t="s">
         <v>168</v>
       </c>
-      <c r="BG11" s="20" t="s">
+      <c r="BG11" s="49" t="s">
         <v>169</v>
       </c>
-      <c r="BH11" s="20" t="s">
+      <c r="BH11" s="49" t="s">
         <v>170</v>
       </c>
-      <c r="BI11" s="20" t="s">
+      <c r="BI11" s="49" t="s">
         <v>171</v>
       </c>
-      <c r="BJ11" s="20" t="s">
+      <c r="BJ11" s="49" t="s">
         <v>172</v>
       </c>
-      <c r="BK11" s="20" t="s">
+      <c r="BK11" s="49" t="s">
         <v>173</v>
       </c>
-      <c r="BL11" s="20" t="s">
+      <c r="BL11" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="BM11" s="20" t="s">
+      <c r="BM11" s="49" t="s">
         <v>175</v>
       </c>
-      <c r="BN11" s="20" t="s">
+      <c r="BN11" s="49" t="s">
         <v>176</v>
       </c>
-      <c r="BO11" s="22" t="s">
+      <c r="BO11" s="50" t="s">
         <v>177</v>
       </c>
-      <c r="BP11" s="20" t="s">
+      <c r="BP11" s="49" t="s">
         <v>178</v>
       </c>
-      <c r="BQ11" s="20" t="s">
+      <c r="BQ11" s="49" t="s">
         <v>179</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="55">
+    <mergeCell ref="BI7:BK7"/>
+    <mergeCell ref="BM7:BM8"/>
+    <mergeCell ref="BN7:BN8"/>
+    <mergeCell ref="BA7:BA8"/>
+    <mergeCell ref="AF7:AI7"/>
+    <mergeCell ref="AJ7:AM7"/>
+    <mergeCell ref="AN7:AQ7"/>
+    <mergeCell ref="AR7:AR8"/>
+    <mergeCell ref="AS7:AT8"/>
+    <mergeCell ref="BL6:BL8"/>
+    <mergeCell ref="BM6:BO6"/>
+    <mergeCell ref="BE7:BE8"/>
+    <mergeCell ref="BF7:BF8"/>
+    <mergeCell ref="BG7:BG8"/>
+    <mergeCell ref="BH7:BH8"/>
+    <mergeCell ref="AU7:AU8"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="AG8:AH8"/>
+    <mergeCell ref="AK8:AL8"/>
+    <mergeCell ref="P7:S7"/>
+    <mergeCell ref="T7:W7"/>
+    <mergeCell ref="AB7:AE7"/>
+    <mergeCell ref="AC8:AD8"/>
+    <mergeCell ref="BB7:BC8"/>
+    <mergeCell ref="BD7:BD8"/>
+    <mergeCell ref="Y8:Z8"/>
+    <mergeCell ref="X7:AA7"/>
+    <mergeCell ref="BP6:BQ7"/>
+    <mergeCell ref="P6:AQ6"/>
+    <mergeCell ref="AR6:AV6"/>
+    <mergeCell ref="AW6:AZ6"/>
+    <mergeCell ref="BA6:BD6"/>
+    <mergeCell ref="BE6:BH6"/>
+    <mergeCell ref="BI6:BK6"/>
+    <mergeCell ref="BO7:BO8"/>
+    <mergeCell ref="AV7:AV8"/>
+    <mergeCell ref="AW7:AW8"/>
+    <mergeCell ref="AX7:AY8"/>
+    <mergeCell ref="AZ7:AZ8"/>
     <mergeCell ref="M8:N8"/>
     <mergeCell ref="B1:O1"/>
     <mergeCell ref="B2:O2"/>
@@ -2773,45 +2803,6 @@
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="J7:J8"/>
-    <mergeCell ref="BB7:BC8"/>
-    <mergeCell ref="BD7:BD8"/>
-    <mergeCell ref="Y8:Z8"/>
-    <mergeCell ref="X7:AA7"/>
-    <mergeCell ref="BP6:BQ7"/>
-    <mergeCell ref="P6:AQ6"/>
-    <mergeCell ref="AR6:AV6"/>
-    <mergeCell ref="AW6:AZ6"/>
-    <mergeCell ref="BA6:BD6"/>
-    <mergeCell ref="BE6:BH6"/>
-    <mergeCell ref="BI6:BK6"/>
-    <mergeCell ref="BO7:BO8"/>
-    <mergeCell ref="AV7:AV8"/>
-    <mergeCell ref="AW7:AW8"/>
-    <mergeCell ref="AX7:AY8"/>
-    <mergeCell ref="AZ7:AZ8"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="AG8:AH8"/>
-    <mergeCell ref="AK8:AL8"/>
-    <mergeCell ref="P7:S7"/>
-    <mergeCell ref="T7:W7"/>
-    <mergeCell ref="AB7:AE7"/>
-    <mergeCell ref="AC8:AD8"/>
-    <mergeCell ref="BI7:BK7"/>
-    <mergeCell ref="BM7:BM8"/>
-    <mergeCell ref="BN7:BN8"/>
-    <mergeCell ref="BA7:BA8"/>
-    <mergeCell ref="AF7:AI7"/>
-    <mergeCell ref="AJ7:AM7"/>
-    <mergeCell ref="AN7:AQ7"/>
-    <mergeCell ref="AR7:AR8"/>
-    <mergeCell ref="AS7:AT8"/>
-    <mergeCell ref="BL6:BL8"/>
-    <mergeCell ref="BM6:BO6"/>
-    <mergeCell ref="BE7:BE8"/>
-    <mergeCell ref="BF7:BF8"/>
-    <mergeCell ref="BG7:BG8"/>
-    <mergeCell ref="BH7:BH8"/>
-    <mergeCell ref="AU7:AU8"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix templates with fixing header
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/summaryReportForm1.xlsx
+++ b/src/main/resources/templates/summaryReportForm1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BCCF2B4-B564-4753-AF38-7FE8D43B770E}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A0BE853-0BF7-4D6E-ABC2-82D7B6E3C37C}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1020,27 +1020,90 @@
     <xf numFmtId="49" fontId="7" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1056,74 +1119,11 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1415,22 +1415,22 @@
   <sheetData>
     <row r="1" spans="1:69" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
       <c r="P1" s="3"/>
       <c r="Q1" s="3"/>
       <c r="R1" s="3"/>
@@ -1488,22 +1488,22 @@
     </row>
     <row r="2" spans="1:69" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="46"/>
+      <c r="L2" s="46"/>
+      <c r="M2" s="46"/>
+      <c r="N2" s="46"/>
+      <c r="O2" s="46"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
@@ -1777,262 +1777,262 @@
       <c r="BQ5" s="2"/>
     </row>
     <row r="6" spans="1:69" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="32" t="s">
+      <c r="E6" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="32" t="s">
+      <c r="F6" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
-      <c r="J6" s="32"/>
-      <c r="K6" s="25" t="s">
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="35" t="s">
         <v>181</v>
       </c>
-      <c r="L6" s="22" t="s">
+      <c r="L6" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="32"/>
-      <c r="N6" s="32"/>
-      <c r="O6" s="32"/>
-      <c r="P6" s="38" t="s">
+      <c r="M6" s="34"/>
+      <c r="N6" s="34"/>
+      <c r="O6" s="34"/>
+      <c r="P6" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="Q6" s="39"/>
-      <c r="R6" s="39"/>
-      <c r="S6" s="39"/>
-      <c r="T6" s="39"/>
-      <c r="U6" s="39"/>
-      <c r="V6" s="39"/>
-      <c r="W6" s="39"/>
-      <c r="X6" s="39"/>
-      <c r="Y6" s="39"/>
-      <c r="Z6" s="39"/>
-      <c r="AA6" s="39"/>
-      <c r="AB6" s="39"/>
-      <c r="AC6" s="39"/>
-      <c r="AD6" s="39"/>
-      <c r="AE6" s="39"/>
-      <c r="AF6" s="39"/>
-      <c r="AG6" s="39"/>
-      <c r="AH6" s="39"/>
-      <c r="AI6" s="39"/>
-      <c r="AJ6" s="39"/>
-      <c r="AK6" s="39"/>
-      <c r="AL6" s="39"/>
-      <c r="AM6" s="39"/>
-      <c r="AN6" s="39"/>
-      <c r="AO6" s="39"/>
-      <c r="AP6" s="39"/>
-      <c r="AQ6" s="39"/>
-      <c r="AR6" s="22" t="s">
+      <c r="Q6" s="42"/>
+      <c r="R6" s="42"/>
+      <c r="S6" s="42"/>
+      <c r="T6" s="42"/>
+      <c r="U6" s="42"/>
+      <c r="V6" s="42"/>
+      <c r="W6" s="42"/>
+      <c r="X6" s="42"/>
+      <c r="Y6" s="42"/>
+      <c r="Z6" s="42"/>
+      <c r="AA6" s="42"/>
+      <c r="AB6" s="42"/>
+      <c r="AC6" s="42"/>
+      <c r="AD6" s="42"/>
+      <c r="AE6" s="42"/>
+      <c r="AF6" s="42"/>
+      <c r="AG6" s="42"/>
+      <c r="AH6" s="42"/>
+      <c r="AI6" s="42"/>
+      <c r="AJ6" s="42"/>
+      <c r="AK6" s="42"/>
+      <c r="AL6" s="42"/>
+      <c r="AM6" s="42"/>
+      <c r="AN6" s="42"/>
+      <c r="AO6" s="42"/>
+      <c r="AP6" s="42"/>
+      <c r="AQ6" s="42"/>
+      <c r="AR6" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="AS6" s="32"/>
-      <c r="AT6" s="32"/>
-      <c r="AU6" s="32"/>
-      <c r="AV6" s="25"/>
-      <c r="AW6" s="40" t="s">
+      <c r="AS6" s="34"/>
+      <c r="AT6" s="34"/>
+      <c r="AU6" s="34"/>
+      <c r="AV6" s="35"/>
+      <c r="AW6" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="AX6" s="32"/>
-      <c r="AY6" s="32"/>
-      <c r="AZ6" s="32"/>
-      <c r="BA6" s="22" t="s">
+      <c r="AX6" s="34"/>
+      <c r="AY6" s="34"/>
+      <c r="AZ6" s="34"/>
+      <c r="BA6" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="BB6" s="32"/>
-      <c r="BC6" s="32"/>
-      <c r="BD6" s="25"/>
-      <c r="BE6" s="41" t="s">
+      <c r="BB6" s="34"/>
+      <c r="BC6" s="34"/>
+      <c r="BD6" s="35"/>
+      <c r="BE6" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="BF6" s="41"/>
-      <c r="BG6" s="41"/>
-      <c r="BH6" s="42"/>
-      <c r="BI6" s="39" t="s">
+      <c r="BF6" s="44"/>
+      <c r="BG6" s="44"/>
+      <c r="BH6" s="45"/>
+      <c r="BI6" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="BJ6" s="39"/>
-      <c r="BK6" s="39"/>
-      <c r="BL6" s="22" t="s">
+      <c r="BJ6" s="42"/>
+      <c r="BK6" s="42"/>
+      <c r="BL6" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="BM6" s="22" t="s">
+      <c r="BM6" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="BN6" s="32"/>
-      <c r="BO6" s="25"/>
-      <c r="BP6" s="32" t="s">
+      <c r="BN6" s="34"/>
+      <c r="BO6" s="35"/>
+      <c r="BP6" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="BQ6" s="32"/>
+      <c r="BQ6" s="34"/>
     </row>
     <row r="7" spans="1:69" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="23"/>
-      <c r="B7" s="26"/>
-      <c r="C7" s="29"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20" t="s">
+      <c r="A7" s="30"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="52"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="33" t="s">
+      <c r="G7" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="H7" s="33" t="s">
+      <c r="H7" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="20" t="s">
+      <c r="I7" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="J7" s="20" t="s">
+      <c r="J7" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="26"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="20"/>
-      <c r="N7" s="20"/>
-      <c r="O7" s="20"/>
-      <c r="P7" s="20" t="s">
+      <c r="K7" s="38"/>
+      <c r="L7" s="30"/>
+      <c r="M7" s="31"/>
+      <c r="N7" s="31"/>
+      <c r="O7" s="31"/>
+      <c r="P7" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="Q7" s="20"/>
-      <c r="R7" s="20"/>
-      <c r="S7" s="20"/>
-      <c r="T7" s="20" t="s">
+      <c r="Q7" s="31"/>
+      <c r="R7" s="31"/>
+      <c r="S7" s="31"/>
+      <c r="T7" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="U7" s="20"/>
-      <c r="V7" s="20"/>
-      <c r="W7" s="20"/>
-      <c r="X7" s="35" t="s">
+      <c r="U7" s="31"/>
+      <c r="V7" s="31"/>
+      <c r="W7" s="31"/>
+      <c r="X7" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="Y7" s="37"/>
-      <c r="Z7" s="37"/>
-      <c r="AA7" s="36"/>
-      <c r="AB7" s="20" t="s">
+      <c r="Y7" s="32"/>
+      <c r="Z7" s="32"/>
+      <c r="AA7" s="40"/>
+      <c r="AB7" s="31" t="s">
         <v>182</v>
       </c>
-      <c r="AC7" s="20"/>
-      <c r="AD7" s="20"/>
-      <c r="AE7" s="20"/>
-      <c r="AF7" s="20" t="s">
+      <c r="AC7" s="31"/>
+      <c r="AD7" s="31"/>
+      <c r="AE7" s="31"/>
+      <c r="AF7" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="AG7" s="20"/>
-      <c r="AH7" s="20"/>
-      <c r="AI7" s="20"/>
-      <c r="AJ7" s="20" t="s">
+      <c r="AG7" s="31"/>
+      <c r="AH7" s="31"/>
+      <c r="AI7" s="31"/>
+      <c r="AJ7" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="AK7" s="20"/>
-      <c r="AL7" s="20"/>
-      <c r="AM7" s="20"/>
-      <c r="AN7" s="37" t="s">
+      <c r="AK7" s="31"/>
+      <c r="AL7" s="31"/>
+      <c r="AM7" s="31"/>
+      <c r="AN7" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="AO7" s="37"/>
-      <c r="AP7" s="37"/>
-      <c r="AQ7" s="37"/>
-      <c r="AR7" s="23" t="s">
+      <c r="AO7" s="32"/>
+      <c r="AP7" s="32"/>
+      <c r="AQ7" s="32"/>
+      <c r="AR7" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="AS7" s="20" t="s">
+      <c r="AS7" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="AT7" s="20"/>
-      <c r="AU7" s="20"/>
-      <c r="AV7" s="26" t="s">
+      <c r="AT7" s="31"/>
+      <c r="AU7" s="31"/>
+      <c r="AV7" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="AW7" s="36" t="s">
+      <c r="AW7" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="AX7" s="20" t="s">
+      <c r="AX7" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="AY7" s="20"/>
-      <c r="AZ7" s="20"/>
-      <c r="BA7" s="23" t="s">
+      <c r="AY7" s="31"/>
+      <c r="AZ7" s="31"/>
+      <c r="BA7" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="BB7" s="20" t="s">
+      <c r="BB7" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="BC7" s="20"/>
-      <c r="BD7" s="26"/>
-      <c r="BE7" s="20" t="s">
+      <c r="BC7" s="31"/>
+      <c r="BD7" s="38"/>
+      <c r="BE7" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="BF7" s="20" t="s">
+      <c r="BF7" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="BG7" s="44" t="s">
+      <c r="BG7" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="BH7" s="45" t="s">
+      <c r="BH7" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="BI7" s="43" t="s">
+      <c r="BI7" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="BJ7" s="43"/>
-      <c r="BK7" s="43"/>
-      <c r="BL7" s="23"/>
-      <c r="BM7" s="23" t="s">
+      <c r="BJ7" s="29"/>
+      <c r="BK7" s="29"/>
+      <c r="BL7" s="30"/>
+      <c r="BM7" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="BN7" s="20" t="s">
+      <c r="BN7" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="BO7" s="26"/>
-      <c r="BP7" s="20"/>
-      <c r="BQ7" s="20"/>
+      <c r="BO7" s="38"/>
+      <c r="BP7" s="31"/>
+      <c r="BQ7" s="31"/>
     </row>
     <row r="8" spans="1:69" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="23"/>
-      <c r="B8" s="26"/>
-      <c r="C8" s="29"/>
+      <c r="A8" s="30"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="50"/>
       <c r="D8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="20"/>
-      <c r="J8" s="20"/>
-      <c r="K8" s="26"/>
+      <c r="E8" s="31"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="54"/>
+      <c r="H8" s="54"/>
+      <c r="I8" s="31"/>
+      <c r="J8" s="31"/>
+      <c r="K8" s="38"/>
       <c r="L8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M8" s="20" t="s">
+      <c r="M8" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="N8" s="20"/>
+      <c r="N8" s="31"/>
       <c r="O8" s="8"/>
       <c r="P8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="Q8" s="20" t="s">
+      <c r="Q8" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="R8" s="20"/>
+      <c r="R8" s="31"/>
       <c r="S8" s="8"/>
       <c r="T8" s="8" t="s">
         <v>19</v>
@@ -2049,34 +2049,34 @@
       <c r="X8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="Y8" s="35" t="s">
+      <c r="Y8" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="Z8" s="36"/>
+      <c r="Z8" s="40"/>
       <c r="AA8" s="8"/>
       <c r="AB8" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="AC8" s="20" t="s">
+      <c r="AC8" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="AD8" s="20"/>
+      <c r="AD8" s="31"/>
       <c r="AE8" s="17"/>
       <c r="AF8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="AG8" s="20" t="s">
+      <c r="AG8" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="AH8" s="20"/>
+      <c r="AH8" s="31"/>
       <c r="AI8" s="8"/>
       <c r="AJ8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="AK8" s="20" t="s">
+      <c r="AK8" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="AL8" s="20"/>
+      <c r="AL8" s="31"/>
       <c r="AM8" s="8"/>
       <c r="AN8" s="8" t="s">
         <v>42</v>
@@ -2090,23 +2090,23 @@
       <c r="AQ8" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="AR8" s="23"/>
-      <c r="AS8" s="20"/>
-      <c r="AT8" s="20"/>
-      <c r="AU8" s="20"/>
-      <c r="AV8" s="26"/>
-      <c r="AW8" s="36"/>
-      <c r="AX8" s="20"/>
-      <c r="AY8" s="20"/>
-      <c r="AZ8" s="20"/>
-      <c r="BA8" s="23"/>
-      <c r="BB8" s="20"/>
-      <c r="BC8" s="20"/>
-      <c r="BD8" s="26"/>
-      <c r="BE8" s="20"/>
-      <c r="BF8" s="20"/>
-      <c r="BG8" s="44"/>
-      <c r="BH8" s="45"/>
+      <c r="AR8" s="30"/>
+      <c r="AS8" s="31"/>
+      <c r="AT8" s="31"/>
+      <c r="AU8" s="31"/>
+      <c r="AV8" s="38"/>
+      <c r="AW8" s="40"/>
+      <c r="AX8" s="31"/>
+      <c r="AY8" s="31"/>
+      <c r="AZ8" s="31"/>
+      <c r="BA8" s="30"/>
+      <c r="BB8" s="31"/>
+      <c r="BC8" s="31"/>
+      <c r="BD8" s="38"/>
+      <c r="BE8" s="31"/>
+      <c r="BF8" s="31"/>
+      <c r="BG8" s="36"/>
+      <c r="BH8" s="37"/>
       <c r="BI8" s="8" t="s">
         <v>46</v>
       </c>
@@ -2116,10 +2116,10 @@
       <c r="BK8" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="BL8" s="23"/>
-      <c r="BM8" s="23"/>
-      <c r="BN8" s="20"/>
-      <c r="BO8" s="26"/>
+      <c r="BL8" s="30"/>
+      <c r="BM8" s="30"/>
+      <c r="BN8" s="31"/>
+      <c r="BO8" s="38"/>
       <c r="BP8" s="8" t="s">
         <v>49</v>
       </c>
@@ -2128,9 +2128,9 @@
       </c>
     </row>
     <row r="9" spans="1:69" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="24"/>
-      <c r="B9" s="27"/>
-      <c r="C9" s="29"/>
+      <c r="A9" s="47"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="50"/>
       <c r="D9" s="10" t="s">
         <v>192</v>
       </c>
@@ -2334,420 +2334,459 @@
       <c r="A10" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="52"/>
-      <c r="C10" s="46" t="s">
+      <c r="B10" s="26"/>
+      <c r="C10" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="D10" s="46" t="s">
+      <c r="D10" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="E10" s="46" t="s">
+      <c r="E10" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="46" t="s">
+      <c r="F10" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="G10" s="46" t="s">
+      <c r="G10" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="H10" s="46" t="s">
+      <c r="H10" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="I10" s="46" t="s">
+      <c r="I10" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="J10" s="46" t="s">
+      <c r="J10" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="K10" s="46" t="s">
+      <c r="K10" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="L10" s="46" t="s">
+      <c r="L10" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="M10" s="46" t="s">
+      <c r="M10" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="N10" s="46" t="s">
+      <c r="N10" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="O10" s="46" t="s">
+      <c r="O10" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="P10" s="46" t="s">
+      <c r="P10" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="Q10" s="46" t="s">
+      <c r="Q10" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="R10" s="46" t="s">
+      <c r="R10" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="S10" s="47" t="s">
+      <c r="S10" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="T10" s="46" t="s">
+      <c r="T10" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="U10" s="46" t="s">
+      <c r="U10" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="V10" s="46" t="s">
+      <c r="V10" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="W10" s="46" t="s">
+      <c r="W10" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="X10" s="46" t="s">
+      <c r="X10" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="Y10" s="46" t="s">
+      <c r="Y10" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="Z10" s="46" t="s">
+      <c r="Z10" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="AA10" s="48" t="s">
+      <c r="AA10" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="AB10" s="46" t="s">
+      <c r="AB10" s="20" t="s">
         <v>183</v>
       </c>
-      <c r="AC10" s="47" t="s">
+      <c r="AC10" s="21" t="s">
         <v>184</v>
       </c>
-      <c r="AD10" s="46" t="s">
+      <c r="AD10" s="20" t="s">
         <v>185</v>
       </c>
-      <c r="AE10" s="47" t="s">
+      <c r="AE10" s="21" t="s">
         <v>190</v>
       </c>
-      <c r="AF10" s="46" t="s">
+      <c r="AF10" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="AG10" s="47" t="s">
+      <c r="AG10" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="AH10" s="46" t="s">
+      <c r="AH10" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="AI10" s="47" t="s">
+      <c r="AI10" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="AJ10" s="46" t="s">
+      <c r="AJ10" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="AK10" s="46" t="s">
+      <c r="AK10" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="AL10" s="46" t="s">
+      <c r="AL10" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="AM10" s="47" t="s">
+      <c r="AM10" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="AN10" s="46" t="s">
+      <c r="AN10" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="AO10" s="46" t="s">
+      <c r="AO10" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="AP10" s="46" t="s">
+      <c r="AP10" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="AQ10" s="46" t="s">
+      <c r="AQ10" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="AR10" s="46" t="s">
+      <c r="AR10" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="AS10" s="46" t="s">
+      <c r="AS10" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="AT10" s="46" t="s">
+      <c r="AT10" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="AU10" s="46" t="s">
+      <c r="AU10" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="AV10" s="46" t="s">
+      <c r="AV10" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="AW10" s="46" t="s">
+      <c r="AW10" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="AX10" s="46" t="s">
+      <c r="AX10" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="AY10" s="46" t="s">
+      <c r="AY10" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="AZ10" s="46" t="s">
+      <c r="AZ10" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="BA10" s="46" t="s">
+      <c r="BA10" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="BB10" s="46" t="s">
+      <c r="BB10" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="BC10" s="46" t="s">
+      <c r="BC10" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="BD10" s="47" t="s">
+      <c r="BD10" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="BE10" s="46" t="s">
+      <c r="BE10" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="BF10" s="46" t="s">
+      <c r="BF10" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="BG10" s="46" t="s">
+      <c r="BG10" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="BH10" s="46" t="s">
+      <c r="BH10" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="BI10" s="46" t="s">
+      <c r="BI10" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="BJ10" s="46" t="s">
+      <c r="BJ10" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="BK10" s="46" t="s">
+      <c r="BK10" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="BL10" s="46" t="s">
+      <c r="BL10" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="BM10" s="46" t="s">
+      <c r="BM10" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="BN10" s="46" t="s">
+      <c r="BN10" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="BO10" s="47" t="s">
+      <c r="BO10" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="BP10" s="46" t="s">
+      <c r="BP10" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="BQ10" s="46" t="s">
+      <c r="BQ10" s="20" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:69" s="16" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="53" t="s">
+      <c r="A11" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="B11" s="54" t="s">
+      <c r="B11" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="C11" s="49" t="s">
+      <c r="C11" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="D11" s="49" t="s">
+      <c r="D11" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="E11" s="49" t="s">
+      <c r="E11" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="F11" s="49" t="s">
+      <c r="F11" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="G11" s="49" t="s">
+      <c r="G11" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="H11" s="49" t="s">
+      <c r="H11" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="I11" s="49" t="s">
+      <c r="I11" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="J11" s="49" t="s">
+      <c r="J11" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="K11" s="49" t="s">
+      <c r="K11" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="L11" s="49" t="s">
+      <c r="L11" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="M11" s="49" t="s">
+      <c r="M11" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="N11" s="49" t="s">
+      <c r="N11" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="O11" s="49" t="s">
+      <c r="O11" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="P11" s="49" t="s">
+      <c r="P11" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="Q11" s="49" t="s">
+      <c r="Q11" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="R11" s="49" t="s">
+      <c r="R11" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="S11" s="50" t="s">
+      <c r="S11" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="T11" s="49" t="s">
+      <c r="T11" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="U11" s="49" t="s">
+      <c r="U11" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="V11" s="49" t="s">
+      <c r="V11" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="W11" s="49" t="s">
+      <c r="W11" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="X11" s="49" t="s">
+      <c r="X11" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="Y11" s="49" t="s">
+      <c r="Y11" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="Z11" s="49" t="s">
+      <c r="Z11" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="AA11" s="51" t="s">
+      <c r="AA11" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="AB11" s="49" t="s">
+      <c r="AB11" s="23" t="s">
         <v>186</v>
       </c>
-      <c r="AC11" s="50" t="s">
+      <c r="AC11" s="24" t="s">
         <v>187</v>
       </c>
-      <c r="AD11" s="49" t="s">
+      <c r="AD11" s="23" t="s">
         <v>188</v>
       </c>
-      <c r="AE11" s="50" t="s">
+      <c r="AE11" s="24" t="s">
         <v>189</v>
       </c>
-      <c r="AF11" s="49" t="s">
+      <c r="AF11" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="AG11" s="50" t="s">
+      <c r="AG11" s="24" t="s">
         <v>142</v>
       </c>
-      <c r="AH11" s="49" t="s">
+      <c r="AH11" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="AI11" s="50" t="s">
+      <c r="AI11" s="24" t="s">
         <v>145</v>
       </c>
-      <c r="AJ11" s="49" t="s">
+      <c r="AJ11" s="23" t="s">
         <v>146</v>
       </c>
-      <c r="AK11" s="49" t="s">
+      <c r="AK11" s="23" t="s">
         <v>147</v>
       </c>
-      <c r="AL11" s="49" t="s">
+      <c r="AL11" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="AM11" s="50" t="s">
+      <c r="AM11" s="24" t="s">
         <v>149</v>
       </c>
-      <c r="AN11" s="49" t="s">
+      <c r="AN11" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="AO11" s="49" t="s">
+      <c r="AO11" s="23" t="s">
         <v>151</v>
       </c>
-      <c r="AP11" s="49" t="s">
+      <c r="AP11" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="AQ11" s="49" t="s">
+      <c r="AQ11" s="23" t="s">
         <v>153</v>
       </c>
-      <c r="AR11" s="49" t="s">
+      <c r="AR11" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="AS11" s="49" t="s">
+      <c r="AS11" s="23" t="s">
         <v>155</v>
       </c>
-      <c r="AT11" s="49" t="s">
+      <c r="AT11" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="AU11" s="49" t="s">
+      <c r="AU11" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="AV11" s="49" t="s">
+      <c r="AV11" s="23" t="s">
         <v>158</v>
       </c>
-      <c r="AW11" s="49" t="s">
+      <c r="AW11" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="AX11" s="49" t="s">
+      <c r="AX11" s="23" t="s">
         <v>160</v>
       </c>
-      <c r="AY11" s="49" t="s">
+      <c r="AY11" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="AZ11" s="49" t="s">
+      <c r="AZ11" s="23" t="s">
         <v>162</v>
       </c>
-      <c r="BA11" s="49" t="s">
+      <c r="BA11" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="BB11" s="49" t="s">
+      <c r="BB11" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="BC11" s="49" t="s">
+      <c r="BC11" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="BD11" s="50" t="s">
+      <c r="BD11" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="BE11" s="49" t="s">
+      <c r="BE11" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="BF11" s="49" t="s">
+      <c r="BF11" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="BG11" s="49" t="s">
+      <c r="BG11" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="BH11" s="49" t="s">
+      <c r="BH11" s="23" t="s">
         <v>170</v>
       </c>
-      <c r="BI11" s="49" t="s">
+      <c r="BI11" s="23" t="s">
         <v>171</v>
       </c>
-      <c r="BJ11" s="49" t="s">
+      <c r="BJ11" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="BK11" s="49" t="s">
+      <c r="BK11" s="23" t="s">
         <v>173</v>
       </c>
-      <c r="BL11" s="49" t="s">
+      <c r="BL11" s="23" t="s">
         <v>174</v>
       </c>
-      <c r="BM11" s="49" t="s">
+      <c r="BM11" s="23" t="s">
         <v>175</v>
       </c>
-      <c r="BN11" s="49" t="s">
+      <c r="BN11" s="23" t="s">
         <v>176</v>
       </c>
-      <c r="BO11" s="50" t="s">
+      <c r="BO11" s="24" t="s">
         <v>177</v>
       </c>
-      <c r="BP11" s="49" t="s">
+      <c r="BP11" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="BQ11" s="49" t="s">
+      <c r="BQ11" s="23" t="s">
         <v>179</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="55">
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="B1:O1"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="F6:J6"/>
+    <mergeCell ref="K6:K8"/>
+    <mergeCell ref="L6:O7"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="BB7:BC8"/>
+    <mergeCell ref="BD7:BD8"/>
+    <mergeCell ref="Y8:Z8"/>
+    <mergeCell ref="X7:AA7"/>
+    <mergeCell ref="BP6:BQ7"/>
+    <mergeCell ref="P6:AQ6"/>
+    <mergeCell ref="AR6:AV6"/>
+    <mergeCell ref="AW6:AZ6"/>
+    <mergeCell ref="BA6:BD6"/>
+    <mergeCell ref="BE6:BH6"/>
+    <mergeCell ref="BI6:BK6"/>
+    <mergeCell ref="BO7:BO8"/>
+    <mergeCell ref="AV7:AV8"/>
+    <mergeCell ref="AW7:AW8"/>
+    <mergeCell ref="AX7:AY8"/>
+    <mergeCell ref="AZ7:AZ8"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="AG8:AH8"/>
+    <mergeCell ref="AK8:AL8"/>
+    <mergeCell ref="P7:S7"/>
+    <mergeCell ref="T7:W7"/>
+    <mergeCell ref="AB7:AE7"/>
+    <mergeCell ref="AC8:AD8"/>
     <mergeCell ref="BI7:BK7"/>
     <mergeCell ref="BM7:BM8"/>
     <mergeCell ref="BN7:BN8"/>
@@ -2764,45 +2803,6 @@
     <mergeCell ref="BG7:BG8"/>
     <mergeCell ref="BH7:BH8"/>
     <mergeCell ref="AU7:AU8"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="AG8:AH8"/>
-    <mergeCell ref="AK8:AL8"/>
-    <mergeCell ref="P7:S7"/>
-    <mergeCell ref="T7:W7"/>
-    <mergeCell ref="AB7:AE7"/>
-    <mergeCell ref="AC8:AD8"/>
-    <mergeCell ref="BB7:BC8"/>
-    <mergeCell ref="BD7:BD8"/>
-    <mergeCell ref="Y8:Z8"/>
-    <mergeCell ref="X7:AA7"/>
-    <mergeCell ref="BP6:BQ7"/>
-    <mergeCell ref="P6:AQ6"/>
-    <mergeCell ref="AR6:AV6"/>
-    <mergeCell ref="AW6:AZ6"/>
-    <mergeCell ref="BA6:BD6"/>
-    <mergeCell ref="BE6:BH6"/>
-    <mergeCell ref="BI6:BK6"/>
-    <mergeCell ref="BO7:BO8"/>
-    <mergeCell ref="AV7:AV8"/>
-    <mergeCell ref="AW7:AW8"/>
-    <mergeCell ref="AX7:AY8"/>
-    <mergeCell ref="AZ7:AZ8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="B1:O1"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="C6:C9"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="F6:J6"/>
-    <mergeCell ref="K6:K8"/>
-    <mergeCell ref="L6:O7"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="J7:J8"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>